<commit_message>
feat(summer-prep/optimization): run all 13 scenarios; fix build-rate feasibility; publish downloads
- Raise max_build_share to values that let retiring 2025 stock be replaced
  (incumbent rebuild ~25%/5-yr step, clean techs 12-20%); audit shows all
  scenarios feasible incl. slow_build (x0.5).
- Handle the central scenario's 'none' param in the scenario loop.
- HiGHS solves all 13 scenarios to optimality; results CSVs + summary JSON
  committed for reproducibility.
- Publish model README, .jl copy and full model zip alongside the xlsx.

Claude-Session: https://claude.ai/code/session_018iLnUHEHLtFhfMwHQmjHMe
</commit_message>
<xml_diff>
--- a/public/data/summer-prep-optimization/industry-optimization-inputs.xlsx
+++ b/public/data/summer-prep-optimization/industry-optimization-inputs.xlsx
@@ -576,9 +576,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -593,9 +591,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
@@ -610,9 +606,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-    </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
@@ -627,9 +621,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-    </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
@@ -644,9 +636,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
@@ -670,9 +660,7 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-    </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
@@ -4523,7 +4511,7 @@
         <v>2025</v>
       </c>
       <c r="I2" s="15" t="n">
-        <v>0.05</v>
+        <v>0.25</v>
       </c>
       <c r="J2" s="15" t="n">
         <v>0</v>
@@ -4569,7 +4557,7 @@
         <v>2030</v>
       </c>
       <c r="I3" s="18" t="n">
-        <v>0.05</v>
+        <v>0.12</v>
       </c>
       <c r="J3" s="18" t="n">
         <v>0.6</v>
@@ -4615,7 +4603,7 @@
         <v>2025</v>
       </c>
       <c r="I4" s="15" t="n">
-        <v>0.08</v>
+        <v>0.15</v>
       </c>
       <c r="J4" s="15" t="n">
         <v>0</v>
@@ -4661,7 +4649,7 @@
         <v>2027</v>
       </c>
       <c r="I5" s="18" t="n">
-        <v>0.06</v>
+        <v>0.15</v>
       </c>
       <c r="J5" s="18" t="n">
         <v>0</v>
@@ -4707,7 +4695,7 @@
         <v>2025</v>
       </c>
       <c r="I6" s="15" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="J6" s="15" t="n">
         <v>0</v>
@@ -4753,7 +4741,7 @@
         <v>2025</v>
       </c>
       <c r="I7" s="18" t="n">
-        <v>0.03</v>
+        <v>0.25</v>
       </c>
       <c r="J7" s="18" t="n">
         <v>0</v>
@@ -4845,7 +4833,7 @@
         <v>2028</v>
       </c>
       <c r="I9" s="18" t="n">
-        <v>0.05</v>
+        <v>0.12</v>
       </c>
       <c r="J9" s="18" t="n">
         <v>0.9</v>
@@ -4891,7 +4879,7 @@
         <v>2025</v>
       </c>
       <c r="I10" s="15" t="n">
-        <v>0.12</v>
+        <v>0.15</v>
       </c>
       <c r="J10" s="15" t="n">
         <v>0</v>
@@ -4937,7 +4925,7 @@
         <v>2025</v>
       </c>
       <c r="I11" s="18" t="n">
-        <v>0.03</v>
+        <v>0.3</v>
       </c>
       <c r="J11" s="18" t="n">
         <v>0</v>
@@ -4983,7 +4971,7 @@
         <v>2030</v>
       </c>
       <c r="I12" s="15" t="n">
-        <v>0.04</v>
+        <v>0.15</v>
       </c>
       <c r="J12" s="15" t="n">
         <v>0</v>
@@ -5029,7 +5017,7 @@
         <v>2027</v>
       </c>
       <c r="I13" s="18" t="n">
-        <v>0.05</v>
+        <v>0.15</v>
       </c>
       <c r="J13" s="18" t="n">
         <v>0</v>
@@ -5075,7 +5063,7 @@
         <v>2032</v>
       </c>
       <c r="I14" s="15" t="n">
-        <v>0.03</v>
+        <v>0.15</v>
       </c>
       <c r="J14" s="15" t="n">
         <v>0.65</v>
@@ -5121,7 +5109,7 @@
         <v>2025</v>
       </c>
       <c r="I15" s="18" t="n">
-        <v>0.05</v>
+        <v>0.3</v>
       </c>
       <c r="J15" s="18" t="n">
         <v>0</v>
@@ -5167,7 +5155,7 @@
         <v>2026</v>
       </c>
       <c r="I16" s="15" t="n">
-        <v>0.06</v>
+        <v>0.15</v>
       </c>
       <c r="J16" s="15" t="n">
         <v>0.6</v>
@@ -5213,7 +5201,7 @@
         <v>2026</v>
       </c>
       <c r="I17" s="18" t="n">
-        <v>0.05</v>
+        <v>0.15</v>
       </c>
       <c r="J17" s="18" t="n">
         <v>0</v>
@@ -5259,7 +5247,7 @@
         <v>2025</v>
       </c>
       <c r="I18" s="15" t="n">
-        <v>0.03</v>
+        <v>0.3</v>
       </c>
       <c r="J18" s="15" t="n">
         <v>0</v>
@@ -5305,7 +5293,7 @@
         <v>2032</v>
       </c>
       <c r="I19" s="18" t="n">
-        <v>0.02</v>
+        <v>0.15</v>
       </c>
       <c r="J19" s="18" t="n">
         <v>0</v>
@@ -5351,7 +5339,7 @@
         <v>2025</v>
       </c>
       <c r="I20" s="15" t="n">
-        <v>0.15</v>
+        <v>0.25</v>
       </c>
       <c r="J20" s="15" t="n">
         <v>0</v>
@@ -5397,7 +5385,7 @@
         <v>2025</v>
       </c>
       <c r="I21" s="18" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="J21" s="18" t="n">
         <v>0</v>
@@ -5443,7 +5431,7 @@
         <v>2025</v>
       </c>
       <c r="I22" s="15" t="n">
-        <v>0.08</v>
+        <v>0.2</v>
       </c>
       <c r="J22" s="15" t="n">
         <v>0</v>
@@ -5489,7 +5477,7 @@
         <v>2027</v>
       </c>
       <c r="I23" s="18" t="n">
-        <v>0.08</v>
+        <v>0.2</v>
       </c>
       <c r="J23" s="18" t="n">
         <v>0</v>
@@ -5535,7 +5523,7 @@
         <v>2025</v>
       </c>
       <c r="I24" s="15" t="n">
-        <v>0.05</v>
+        <v>0.25</v>
       </c>
       <c r="J24" s="15" t="n">
         <v>0</v>
@@ -5581,7 +5569,7 @@
         <v>2027</v>
       </c>
       <c r="I25" s="18" t="n">
-        <v>0.08</v>
+        <v>0.15</v>
       </c>
       <c r="J25" s="18" t="n">
         <v>0</v>
@@ -5627,7 +5615,7 @@
         <v>2025</v>
       </c>
       <c r="I26" s="15" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="J26" s="15" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
feat(summer-prep/optimization): make the DEA Technology Data Catalogue the primary data source
Downloaded and read the Danish Energy Agency datasheets (Industrial Process
Heat, Carbon Capture Transport & Storage, Renewable Fuels) and re-grounded
the CCS add-ons, process-heat electrification/biomass techs, electrolytic
ammonia and the hydrogen price path in them, with documented unit
conversions per row and verified ens.dk links. Fixes an electrolyser
double-count in the old ammonia_h2 capex. Non-DEA-covered equipment
(BF-BOF, DRI, kilns, crackers, smelters, SMR) keeps IEA/literature sources.
All 13 scenarios re-solved to optimality; DEA-based hydrogen prices push
H2-DRI/e-ammonia out of the central case (they enter only under h2_cheap).
Workbook, JSON/TS mirrors and zip regenerated.

Claude-Session: https://claude.ai/code/session_018iLnUHEHLtFhfMwHQmjHMe
</commit_message>
<xml_diff>
--- a/public/data/summer-prep-optimization/industry-optimization-inputs.xlsx
+++ b/public/data/summer-prep-optimization/industry-optimization-inputs.xlsx
@@ -29,7 +29,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Emission Factors'!$A$1:$E$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Constraints'!$A$1:$F$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Scenarios'!$A$1:$F$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Sources'!$A$1:$G$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Sources'!$A$1:$G$80</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -575,7 +575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -628,14 +628,14 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Scope &amp; geography</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="70" customHeight="1">
+          <t>Primary data source</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="140" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Geography: EU-27. Subsectors: steel (crude steel, integrated + EAF routes), cement (clinker-based), high-value chemicals / HVC (steam cracking: ethylene, propylene, aromatics), ammonia, aluminium (primary + secondary), glass (container &amp; flat) and pulp &amp; paper. The subsector/technology/carrier/scenario identifiers used throughout this workbook and the underlying model code are fixed and must not be renamed.</t>
+          <t>The Danish Energy Agency (DEA) Technology Data catalogue series (ens.dk/en/analyses-and-statistics/technology-data) is the primary data source for this model wherever it plausibly covers the underlying equipment: Technology Data for Carbon Capture, Transport and Storage grounds every CCS variant's capture capex, O&amp;M and lifetime; Technology Data for Industrial Process Heat grounds electrification (heat pumps, direct electric firing) and biomass/alternative-fuel process-heat technologies in paper, glass and cement; Technology Data for Renewable Fuels grounds the electrolytic-hydrogen ammonia route and the hydrogen price path used throughout the model. Where DEA genuinely has no coverage — blast-furnace/DRI/EAF steel metallurgy, cement clinker kilns, steam crackers, aluminium smelting, SMR reforming — the pre-existing IEA/IEAGHG/JRC/etc. literature remains primary: DEA is the primary source, not the exclusive one. See the 'sources' sheet for the full register, including a summary row (table=technologies, item=multiple) explaining this policy, and each affected row's 'source' cell for the specific DEA datasheet and conversion used.</t>
         </is>
       </c>
     </row>
@@ -645,14 +645,14 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Units</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="140" customHeight="1">
+          <t>Scope &amp; geography</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="70" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Production &amp; demand: Mt product/yr. CAPEX: EUR per tonne/yr of installed capacity. Fixed OPEX: EUR per tonne/yr of capacity, per year. Variable (non-energy) OPEX: EUR per tonne of product (feedstock, consumables, labour — excludes fuel &amp; carbon cost, which are computed from the energy-use and price tables). Energy use: GJ per tonne of product, by carrier (coal, coke, natural gas, electricity, hydrogen, biomass, oil). Fuel &amp; electricity prices: EUR per GJ (multiply by 3.6 to convert EUR/MWh &lt;-&gt; EUR/GJ for electricity and hydrogen). Carbon price: EUR per tonne of CO2 (EU ETS path). Emission factors: tonnes CO2 per GJ of fuel (combustion factors; the electricity factor is the EU-27 grid emission intensity and varies by year as the grid decarbonises). Process CO2: tonnes CO2 per tonne of product, non-energy chemistry (e.g. limestone calcination in cement, anode consumption in aluminium) not captured by fuel combustion factors. Capture rate: share of a technology's CO2 captured by CCS (0 for technologies without CCS).</t>
+          <t>Geography: EU-27. Subsectors: steel (crude steel, integrated + EAF routes), cement (clinker-based), high-value chemicals / HVC (steam cracking: ethylene, propylene, aromatics), ammonia, aluminium (primary + secondary), glass (container &amp; flat) and pulp &amp; paper. The subsector/technology/carrier/scenario identifiers used throughout this workbook and the underlying model code are fixed and must not be renamed.</t>
         </is>
       </c>
     </row>
@@ -662,12 +662,29 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
+          <t>Units</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="140" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Production &amp; demand: Mt product/yr. CAPEX: EUR per tonne/yr of installed capacity. Fixed OPEX: EUR per tonne/yr of capacity, per year. Variable (non-energy) OPEX: EUR per tonne of product (feedstock, consumables, labour — excludes fuel &amp; carbon cost, which are computed from the energy-use and price tables). Energy use: GJ per tonne of product, by carrier (coal, coke, natural gas, electricity, hydrogen, biomass, oil). Fuel &amp; electricity prices: EUR per GJ (multiply by 3.6 to convert EUR/MWh &lt;-&gt; EUR/GJ for electricity and hydrogen). Carbon price: EUR per tonne of CO2 (EU ETS path). Emission factors: tonnes CO2 per GJ of fuel (combustion factors; the electricity factor is the EU-27 grid emission intensity and varies by year as the grid decarbonises). Process CO2: tonnes CO2 per tonne of product, non-energy chemistry (e.g. limestone calcination in cement, anode consumption in aluminium) not captured by fuel combustion factors. Capture rate: share of a technology's CO2 captured by CCS (0 for technologies without CCS).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>How the sheets relate</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="180" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="19" ht="180" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>sectors — one row per subsector with 2023 production and direct CO2 anchors.
 demand — the central demand path per subsector and model year (sensitivity scenarios scale this).
@@ -682,35 +699,35 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Per-row sourcing</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="110" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Every data sheet (all except 'sources') carries 'source' and 'source_url' as its last two columns: 'source' is a short citation (Org (Year), Title) and 'source_url' is one working link, wherever possible deep-linking to the exact report or dataset page the number came from (clickable in this sheet). Rows that are genuine modelling choices rather than literature values say so honestly: 'Derived from &lt;source&gt;' for demand paths and the carbon price low/high bands built around a sourced central path, and 'Model assumption (prototype)' for the 13 sensitivity-scenario multipliers in the 'scenarios' sheet, whose source_url points to this model's own README rather than an invented external reference. The 'sources' sheet remains the master register of every citation used, including secondary/cross-check sources not selected as a given row's primary link.</t>
-        </is>
-      </c>
-    </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
+          <t>Per-row sourcing</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="110" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Every data sheet (all except 'sources') carries 'source' and 'source_url' as its last two columns: 'source' is a short citation (Org (Year), Title) and 'source_url' is one working link, wherever possible deep-linking to the exact report or dataset page the number came from (clickable in this sheet). Rows that are genuine modelling choices rather than literature values say so honestly: 'Derived from &lt;source&gt;' for demand paths and the carbon price low/high bands built around a sourced central path, and 'Model assumption (prototype)' for the 13 sensitivity-scenario multipliers in the 'scenarios' sheet, whose source_url points to this model's own README rather than an invented external reference. The 'sources' sheet remains the master register of every citation used, including secondary/cross-check sources not selected as a given row's primary link.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
           <t>Model &amp; downloads</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="60" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="25" ht="60" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>The optimization model itself (Julia + JuMP/HiGHS) lives in the ESABCCMethodHub repo under beta/modules/summer-prep/optimization/model/, in the spirit of the SEAMAPS model (https://github.com/SebastianFra/SEAMAPS). This workbook, the Julia source and the full model bundle (code + data + results + README) are available for download from the 'Summer Prep — Industry Optimization' page of the ESABCC Method Hub.</t>
         </is>
@@ -1172,7 +1189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G73"/>
+  <dimension ref="A1:G80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1747,32 +1764,32 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>steel_bfbof_ccs</t>
+          <t>steel_ngdri_eaf</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>IEAGHG</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Cost of CO2 capture in the industrial sector: cement and iron &amp; steel industries (2018-TR03)</t>
+          <t>Iron and Steel Technology Roadmap</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>https://ieaghg.org/publications/cost-of-co2-capture-in-the-industrial-sector-cement-and-iron-and-steel-industries/</t>
+          <t>https://www.iea.org/reports/iron-and-steel-technology-roadmap</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>Capture-rate and capex premium for BF-BOF + CCUS</t>
+          <t>NG-DRI+EAF energy use and transitional-asset characterisation</t>
         </is>
       </c>
     </row>
@@ -1784,32 +1801,32 @@
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>steel_ngdri_eaf</t>
+          <t>steel_h2dri_eaf</t>
         </is>
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>European Parliament (EPRS)</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>Iron and Steel Technology Roadmap</t>
+          <t>Carbon-free steel production - Cost reduction options and usage of existing gas infrastructure</t>
         </is>
       </c>
       <c r="E17" s="13" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/iron-and-steel-technology-roadmap</t>
+          <t>https://www.europarl.europa.eu/RegData/etudes/STUD/2021/690008/EPRS_STU(2021)690008_EN.pdf</t>
         </is>
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="G17" s="11" t="inlineStr">
         <is>
-          <t>NG-DRI+EAF energy use and transitional-asset characterisation</t>
+          <t>H2-DRI+EAF hydrogen intensity (~50-60 kg H2/t) and MAC ~EUR73-166/tCO2 by 2030</t>
         </is>
       </c>
     </row>
@@ -1826,27 +1843,27 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>European Parliament (EPRS)</t>
+          <t>LeadIT (SEI)</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Carbon-free steel production - Cost reduction options and usage of existing gas infrastructure</t>
+          <t>Green Steel Tracker</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>https://www.europarl.europa.eu/RegData/etudes/STUD/2021/690008/EPRS_STU(2021)690008_EN.pdf</t>
+          <t>https://www.industrytransition.org/green-steel-tracker/</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>H2-DRI+EAF hydrogen intensity (~50-60 kg H2/t) and MAC ~EUR73-166/tCO2 by 2030</t>
+          <t>Commercial availability timeline (first plants building now)</t>
         </is>
       </c>
     </row>
@@ -1858,32 +1875,32 @@
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>steel_h2dri_eaf</t>
+          <t>steel_scrap_eaf</t>
         </is>
       </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>LeadIT (SEI)</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>Green Steel Tracker</t>
+          <t>Iron and Steel Technology Roadmap</t>
         </is>
       </c>
       <c r="E19" s="13" t="inlineStr">
         <is>
-          <t>https://www.industrytransition.org/green-steel-tracker/</t>
+          <t>https://www.iea.org/reports/iron-and-steel-technology-roadmap</t>
         </is>
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="G19" s="11" t="inlineStr">
         <is>
-          <t>Commercial availability timeline (first plants building now)</t>
+          <t>Scrap-EAF as mature, low direct-CO2 route</t>
         </is>
       </c>
     </row>
@@ -1900,27 +1917,27 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>Material Economics</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Iron and Steel Technology Roadmap</t>
+          <t>Industrial Transformation 2050 - Pathways to Net-Zero Emissions from EU Heavy Industry</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/iron-and-steel-technology-roadmap</t>
+          <t>https://materialeconomics.com/sites/default/files/2024-06/material-economics-industrial-transformation-2050-executive-summary.pdf</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>Scrap-EAF as mature, low direct-CO2 route</t>
+          <t>Scrap availability as the binding long-run constraint on secondary steel</t>
         </is>
       </c>
     </row>
@@ -1932,32 +1949,32 @@
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>steel_scrap_eaf</t>
+          <t>cement_ref</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>Material Economics</t>
+          <t>IEA / CSI</t>
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>Industrial Transformation 2050 - Pathways to Net-Zero Emissions from EU Heavy Industry</t>
+          <t>Technology Roadmap: Low-Carbon Transition in the Cement Industry</t>
         </is>
       </c>
       <c r="E21" s="13" t="inlineStr">
         <is>
-          <t>https://materialeconomics.com/sites/default/files/2024-06/material-economics-industrial-transformation-2050-executive-summary.pdf</t>
+          <t>https://www.iea.org/reports/technology-roadmap-low-carbon-transition-in-the-cement-industry</t>
         </is>
       </c>
       <c r="F21" s="10" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2018</t>
         </is>
       </c>
       <c r="G21" s="11" t="inlineStr">
         <is>
-          <t>Scrap availability as the binding long-run constraint on secondary steel</t>
+          <t>Reference kiln thermal energy (~3.4 GJ/t clinker) and clinker-ratio-driven process CO2 (0.53 tCO2/t clinker x 0.77 ratio)</t>
         </is>
       </c>
     </row>
@@ -1969,32 +1986,32 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>cement_ref</t>
+          <t>cement_clinkersub</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>IEA / CSI</t>
+          <t>MDPI (Sustainability, peer-reviewed)</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Technology Roadmap: Low-Carbon Transition in the Cement Industry</t>
+          <t>Limestone Calcined Clay Cement (LC3): From Laboratory Innovation to Sustainable Industrial Application</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/technology-roadmap-low-carbon-transition-in-the-cement-industry</t>
+          <t>https://www.mdpi.com/2071-1050/18/7/3473</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>Reference kiln thermal energy (~3.4 GJ/t clinker) and clinker-ratio-driven process CO2 (0.53 tCO2/t clinker x 0.77 ratio)</t>
+          <t>LC3 clinker replacement up to ~50%, ~40% CO2 cut, near-cost-neutral</t>
         </is>
       </c>
     </row>
@@ -2006,32 +2023,32 @@
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>cement_clinkersub</t>
+          <t>cement_ccs</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>MDPI (Sustainability, peer-reviewed)</t>
+          <t>Heidelberg Materials</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>Limestone Calcined Clay Cement (LC3): From Laboratory Innovation to Sustainable Industrial Application</t>
+          <t>World premiere: CCS cement facility opens in Norway (Brevik CCS)</t>
         </is>
       </c>
       <c r="E23" s="13" t="inlineStr">
         <is>
-          <t>https://www.mdpi.com/2071-1050/18/7/3473</t>
+          <t>https://www.heidelbergmaterials.com/en/pr-2025-06-18</t>
         </is>
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="G23" s="11" t="inlineStr">
         <is>
-          <t>LC3 clinker replacement up to ~50%, ~40% CO2 cut, near-cost-neutral</t>
+          <t>First industrial-scale cement CCS operational since 2025; available_from calibrated to this</t>
         </is>
       </c>
     </row>
@@ -2043,22 +2060,22 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>cement_ccs</t>
+          <t>cement_altfuel</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>IEAGHG</t>
+          <t>IEA / CSI</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Cost of CO2 capture in the industrial sector: cement and iron &amp; steel industries (2018-TR03)</t>
+          <t>Technology Roadmap: Low-Carbon Transition in the Cement Industry</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>https://ieaghg.org/publications/cost-of-co2-capture-in-the-industrial-sector-cement-and-iron-and-steel-industries/</t>
+          <t>https://www.iea.org/reports/technology-roadmap-low-carbon-transition-in-the-cement-industry</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
@@ -2068,7 +2085,7 @@
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>MAC EUR30-107/tCO2 avoided; capture rate ~90% assumed for post-combustion</t>
+          <t>Alternative-fuel co-processing mature and widely deployed</t>
         </is>
       </c>
     </row>
@@ -2080,32 +2097,32 @@
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>cement_ccs</t>
+          <t>hvc_ref</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>Heidelberg Materials</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>World premiere: CCS cement facility opens in Norway (Brevik CCS)</t>
+          <t>The Future of Petrochemicals</t>
         </is>
       </c>
       <c r="E25" s="13" t="inlineStr">
         <is>
-          <t>https://www.heidelbergmaterials.com/en/pr-2025-06-18</t>
+          <t>https://www.iea.org/reports/the-future-of-petrochemicals</t>
         </is>
       </c>
       <c r="F25" s="10" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2018</t>
         </is>
       </c>
       <c r="G25" s="11" t="inlineStr">
         <is>
-          <t>First industrial-scale cement CCS operational since 2025; available_from calibrated to this</t>
+          <t>Reference steam-cracker furnace energy intensity order of magnitude</t>
         </is>
       </c>
     </row>
@@ -2117,32 +2134,32 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>cement_altfuel</t>
+          <t>hvc_elec</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>IEA / CSI</t>
+          <t>BASF / SABIC / Linde</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Technology Roadmap: Low-Carbon Transition in the Cement Industry</t>
+          <t>Start-up of the world's first large-scale electrically heated steam cracking furnace</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/technology-roadmap-low-carbon-transition-in-the-cement-industry</t>
+          <t>https://www.basf.com/global/en/media/news-releases/2024/04/p-24-177</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>Alternative-fuel co-processing mature and widely deployed</t>
+          <t>Electric cracker demonstration; furnace CO2 cut up to ~90%</t>
         </is>
       </c>
     </row>
@@ -2154,7 +2171,7 @@
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>hvc_ref</t>
+          <t>hvc_bio</t>
         </is>
       </c>
       <c r="C27" s="10" t="inlineStr">
@@ -2179,7 +2196,7 @@
       </c>
       <c r="G27" s="11" t="inlineStr">
         <is>
-          <t>Reference steam-cracker furnace energy intensity order of magnitude</t>
+          <t>Bio-naphtha as drop-in feedstock displacing fossil naphtha</t>
         </is>
       </c>
     </row>
@@ -2191,32 +2208,32 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>hvc_elec</t>
+          <t>ammonia_smr</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>BASF / SABIC / Linde</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Start-up of the world's first large-scale electrically heated steam cracking furnace</t>
+          <t>Ammonia Technology Roadmap</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>https://www.basf.com/global/en/media/news-releases/2024/04/p-24-177</t>
+          <t>https://www.iea.org/reports/ammonia-technology-roadmap</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>Electric cracker demonstration; furnace CO2 cut up to ~90%</t>
+          <t>Reference SMR-Haber-Bosch natural gas intensity ~28-32 GJ/t NH3</t>
         </is>
       </c>
     </row>
@@ -2228,32 +2245,32 @@
       </c>
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>hvc_bio</t>
+          <t>ammonia_h2</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>Yara International</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>The Future of Petrochemicals</t>
+          <t>Yara opens renewable hydrogen plant: a major milestone</t>
         </is>
       </c>
       <c r="E29" s="13" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/the-future-of-petrochemicals</t>
+          <t>https://www.yara.com/corporate-releases/yara-opens-renewable-hydrogen-plant-a-major-milestone/</t>
         </is>
       </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="G29" s="11" t="inlineStr">
         <is>
-          <t>Bio-naphtha as drop-in feedstock displacing fossil naphtha</t>
+          <t>First commercial green-ammonia plant (Heroya) inaugurated 2024; calibrates available_from</t>
         </is>
       </c>
     </row>
@@ -2265,32 +2282,32 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>hvc_ccs</t>
+          <t>alu_ref</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>IEAGHG</t>
+          <t>JRC (European Commission)</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Cost of CO2 capture in the industrial sector: cement and iron &amp; steel industries (2018-TR03)</t>
+          <t>Aluminium factsheet (JRC144120)</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>https://ieaghg.org/publications/cost-of-co2-capture-in-the-industrial-sector-cement-and-iron-and-steel-industries/</t>
+          <t>https://publications.jrc.ec.europa.eu/repository/bitstream/JRC144120/Aluminium_factsheet_JRC144120.pdf</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>Industrial CCS cost/capture-rate benchmarks applied to chemicals furnaces (moderate capture, dilute flue gas)</t>
+          <t>Direct anode process CO2 ~1.4 tCO2/t primary Al implied by ~2.75 Mt / ~2 Mt production</t>
         </is>
       </c>
     </row>
@@ -2302,32 +2319,32 @@
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>ammonia_smr</t>
+          <t>alu_ref</t>
         </is>
       </c>
       <c r="C31" s="10" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>International Aluminium Institute (IAI)</t>
         </is>
       </c>
       <c r="D31" s="11" t="inlineStr">
         <is>
-          <t>Ammonia Technology Roadmap</t>
+          <t>Statistics</t>
         </is>
       </c>
       <c r="E31" s="13" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/ammonia-technology-roadmap</t>
+          <t>https://international-aluminium.org/statistics/</t>
         </is>
       </c>
       <c r="F31" s="10" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="G31" s="11" t="inlineStr">
         <is>
-          <t>Reference SMR-Haber-Bosch natural gas intensity ~28-32 GJ/t NH3</t>
+          <t>Primary smelting electricity intensity ~14-15 MWh/t (~51 GJ/t)</t>
         </is>
       </c>
     </row>
@@ -2339,32 +2356,32 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>ammonia_smr_ccs</t>
+          <t>alu_inert</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>ELYSIS</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>Ammonia Technology Roadmap</t>
+          <t>ELYSIS achieves breakthrough with commercial-size cell</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/ammonia-technology-roadmap</t>
+          <t>https://elysis.com/en/elysis-achieves-breakthrough-with-commercial-size-cell-a-first-in-aluminium-production-using-the</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>Blue-ammonia (SMR/ATR+CCS) capture rate and capex premium</t>
+          <t>Full-scale 450 kA commercial-size inert-anode cell started up Nov 2025; eliminates direct process CO2</t>
         </is>
       </c>
     </row>
@@ -2376,32 +2393,32 @@
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>ammonia_h2</t>
+          <t>alu_sec</t>
         </is>
       </c>
       <c r="C33" s="10" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>Material Economics</t>
         </is>
       </c>
       <c r="D33" s="11" t="inlineStr">
         <is>
-          <t>Ammonia Technology Roadmap - Executive Summary</t>
+          <t>Industrial Transformation 2050 - Pathways to Net-Zero Emissions from EU Heavy Industry</t>
         </is>
       </c>
       <c r="E33" s="13" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/ammonia-technology-roadmap/executive-summary</t>
+          <t>https://materialeconomics.com/sites/default/files/2024-06/material-economics-industrial-transformation-2050-executive-summary.pdf</t>
         </is>
       </c>
       <c r="F33" s="10" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="G33" s="11" t="inlineStr">
         <is>
-          <t>Electrolytic-H2 ammonia MAC ~US$820/t NH3 (~US$400/t above conventional); needs power &lt;~US$40/MWh for parity</t>
+          <t>Secondary aluminium uses ~5% of primary smelting energy; scrap-supply constrained</t>
         </is>
       </c>
     </row>
@@ -2413,32 +2430,32 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>ammonia_h2</t>
+          <t>glass_ng</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Yara International</t>
+          <t>European Commission (CINEA)</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>Yara opens renewable hydrogen plant: a major milestone</t>
+          <t>How LIFE is reducing emissions from glass production</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>https://www.yara.com/corporate-releases/yara-opens-renewable-hydrogen-plant-a-major-milestone/</t>
+          <t>https://cinea.ec.europa.eu/news-events/news/how-life-reducing-emissions-glass-production-2022-03-16_en</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>First commercial green-ammonia plant (Heroya) inaugurated 2024; calibrates available_from</t>
+          <t>Reference gas-fired melting energy ~5-7 GJ/t and process CO2 from carbonate raw materials</t>
         </is>
       </c>
     </row>
@@ -2450,32 +2467,32 @@
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>alu_ref</t>
+          <t>glass_elec</t>
         </is>
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>JRC (European Commission)</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="D35" s="11" t="inlineStr">
         <is>
-          <t>Aluminium factsheet (JRC144120)</t>
+          <t>ETP Clean Energy Technology Guide (technology readiness levels)</t>
         </is>
       </c>
       <c r="E35" s="13" t="inlineStr">
         <is>
-          <t>https://publications.jrc.ec.europa.eu/repository/bitstream/JRC144120/Aluminium_factsheet_JRC144120.pdf</t>
+          <t>https://www.iea.org/data-and-statistics/data-tools/etp-clean-energy-technology-guide</t>
         </is>
       </c>
       <c r="F35" s="10" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="G35" s="11" t="inlineStr">
         <is>
-          <t>Direct anode process CO2 ~1.4 tCO2/t primary Al implied by ~2.75 Mt / ~2 Mt production</t>
+          <t>All-electric melting TRL and availability</t>
         </is>
       </c>
     </row>
@@ -2487,22 +2504,22 @@
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>alu_ref</t>
+          <t>glass_hybrid</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>International Aluminium Institute (IAI)</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>Statistics</t>
+          <t>ETP Clean Energy Technology Guide (technology readiness levels)</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>https://international-aluminium.org/statistics/</t>
+          <t>https://www.iea.org/data-and-statistics/data-tools/etp-clean-energy-technology-guide</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
@@ -2512,7 +2529,7 @@
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>Primary smelting electricity intensity ~14-15 MWh/t (~51 GJ/t)</t>
+          <t>Large hybrid furnace TRL 6-8, emerging</t>
         </is>
       </c>
     </row>
@@ -2524,118 +2541,118 @@
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>alu_inert</t>
+          <t>paper_ref</t>
         </is>
       </c>
       <c r="C37" s="10" t="inlineStr">
         <is>
-          <t>ELYSIS</t>
+          <t>CEPI</t>
         </is>
       </c>
       <c r="D37" s="11" t="inlineStr">
         <is>
-          <t>ELYSIS achieves breakthrough with commercial-size cell</t>
+          <t>Key Statistics 2022 - European pulp &amp; paper industry</t>
         </is>
       </c>
       <c r="E37" s="13" t="inlineStr">
         <is>
-          <t>https://elysis.com/en/elysis-achieves-breakthrough-with-commercial-size-cell-a-first-in-aluminium-production-using-the</t>
+          <t>https://www.cepi.org/wp-content/uploads/2023/07/2022-Key-Statistics-FINAL.pdf</t>
         </is>
       </c>
       <c r="F37" s="10" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="G37" s="11" t="inlineStr">
         <is>
-          <t>Full-scale 450 kA commercial-size inert-anode cell started up Nov 2025; eliminates direct process CO2</t>
+          <t>Reference fossil process-heat intensity order of magnitude</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>technologies</t>
+          <t>fuel_prices</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>alu_sec</t>
+          <t>coal</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Material Economics</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>Industrial Transformation 2050 - Pathways to Net-Zero Emissions from EU Heavy Industry</t>
+          <t>World Energy Outlook 2024</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>https://materialeconomics.com/sites/default/files/2024-06/material-economics-industrial-transformation-2050-executive-summary.pdf</t>
+          <t>https://www.iea.org/reports/world-energy-outlook-2024</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>Secondary aluminium uses ~5% of primary smelting energy; scrap-supply constrained</t>
+          <t>Steam coal industrial price path, central scenario order of magnitude ~EUR3/GJ</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="10" t="inlineStr">
         <is>
-          <t>technologies</t>
+          <t>fuel_prices</t>
         </is>
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>glass_ng</t>
+          <t>coke</t>
         </is>
       </c>
       <c r="C39" s="10" t="inlineStr">
         <is>
-          <t>European Commission (CINEA)</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="D39" s="11" t="inlineStr">
         <is>
-          <t>How LIFE is reducing emissions from glass production</t>
+          <t>World Energy Outlook 2024</t>
         </is>
       </c>
       <c r="E39" s="13" t="inlineStr">
         <is>
-          <t>https://cinea.ec.europa.eu/news-events/news/how-life-reducing-emissions-glass-production-2022-03-16_en</t>
+          <t>https://www.iea.org/reports/world-energy-outlook-2024</t>
         </is>
       </c>
       <c r="F39" s="10" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="G39" s="11" t="inlineStr">
         <is>
-          <t>Reference gas-fired melting energy ~5-7 GJ/t and process CO2 from carbonate raw materials</t>
+          <t>Metallurgical coke priced at a premium to thermal coal (~2x)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>technologies</t>
+          <t>fuel_prices</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>glass_elec</t>
+          <t>natural_gas</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
@@ -2645,12 +2662,12 @@
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>ETP Clean Energy Technology Guide (technology readiness levels)</t>
+          <t>World Energy Outlook 2024</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>https://www.iea.org/data-and-statistics/data-tools/etp-clean-energy-technology-guide</t>
+          <t>https://www.iea.org/reports/world-energy-outlook-2024</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
@@ -2660,34 +2677,34 @@
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>All-electric melting TRL and availability</t>
+          <t>EU industrial natural gas price path, central scenario, declining from ~EUR10/GJ (2025)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="10" t="inlineStr">
         <is>
-          <t>technologies</t>
+          <t>fuel_prices</t>
         </is>
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>glass_hybrid</t>
+          <t>electricity</t>
         </is>
       </c>
       <c r="C41" s="10" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>Eurostat</t>
         </is>
       </c>
       <c r="D41" s="11" t="inlineStr">
         <is>
-          <t>ETP Clean Energy Technology Guide (technology readiness levels)</t>
+          <t>Electricity price statistics</t>
         </is>
       </c>
       <c r="E41" s="13" t="inlineStr">
         <is>
-          <t>https://www.iea.org/data-and-statistics/data-tools/etp-clean-energy-technology-guide</t>
+          <t>https://ec.europa.eu/eurostat/statistics-explained/index.php?title=Electricity_price_statistics</t>
         </is>
       </c>
       <c r="F41" s="10" t="inlineStr">
@@ -2697,34 +2714,34 @@
       </c>
       <c r="G41" s="11" t="inlineStr">
         <is>
-          <t>Large hybrid furnace TRL 6-8, emerging</t>
+          <t>EU-27 industrial electricity price ~EUR24/GJ (~EUR86/MWh) in 2025, declining as renewables share rises</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>technologies</t>
+          <t>fuel_prices</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>paper_ref</t>
+          <t>biomass</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>CEPI</t>
+          <t>IEA Bioenergy</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>Key Statistics 2022 - European pulp &amp; paper industry</t>
+          <t>Decarbonizing industrial process heat: the role of biomass</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>https://www.cepi.org/wp-content/uploads/2023/07/2022-Key-Statistics-FINAL.pdf</t>
+          <t>https://www.ieabioenergy.com/blog/publications/decarbonizing-industrial-process-heat-the-role-of-biomass/</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
@@ -2734,19 +2751,19 @@
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>Reference fossil process-heat intensity order of magnitude</t>
+          <t>Solid biomass/residue fuel price order of magnitude ~EUR8/GJ</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="10" t="inlineStr">
         <is>
-          <t>technologies</t>
+          <t>fuel_prices</t>
         </is>
       </c>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>paper_elec</t>
+          <t>oil</t>
         </is>
       </c>
       <c r="C43" s="10" t="inlineStr">
@@ -2756,271 +2773,271 @@
       </c>
       <c r="D43" s="11" t="inlineStr">
         <is>
-          <t>The Future of Heat Pumps</t>
+          <t>World Energy Outlook 2024</t>
         </is>
       </c>
       <c r="E43" s="13" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/the-future-of-heat-pumps</t>
+          <t>https://www.iea.org/reports/world-energy-outlook-2024</t>
         </is>
       </c>
       <c r="F43" s="10" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="G43" s="11" t="inlineStr">
         <is>
-          <t>Industrial heat-pump electrification of process heat; TRL and availability</t>
+          <t>Industrial oil/naphtha price path, central scenario order of magnitude ~EUR14/GJ</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>technologies</t>
+          <t>carbon_price</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>paper_bio</t>
+          <t>eu_ets</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>IEA Bioenergy</t>
+          <t>European Commission (DG CLIMA)</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>Decarbonizing industrial process heat: the role of biomass</t>
+          <t>2040 Climate Target</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>https://www.ieabioenergy.com/blog/publications/decarbonizing-industrial-process-heat-the-role-of-biomass/</t>
+          <t>https://commission.europa.eu/topics/climate-action/eu-climate-energy-and-environmental-targets/2040-targets_en</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>Biomass/black-liquor process heat, commercially mature</t>
+          <t>Central EU ETS price path ~EUR80/t (2025) rising to ~EUR200/t (2040) and ~EUR250/t (2050); low/high bands constructed around this by the model team, consistent with the range of EC impact-assessment and market-forward modelling</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>fuel_prices</t>
+          <t>carbon_price</t>
         </is>
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>coal</t>
+          <t>eu_ets</t>
         </is>
       </c>
       <c r="C45" s="10" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>ICAP</t>
         </is>
       </c>
       <c r="D45" s="11" t="inlineStr">
         <is>
-          <t>World Energy Outlook 2024</t>
+          <t>EU Emissions Trading System (EU ETS)</t>
         </is>
       </c>
       <c r="E45" s="13" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/world-energy-outlook-2024</t>
+          <t>https://icapcarbonaction.com/en/ets/eu-emissions-trading-system-eu-ets</t>
         </is>
       </c>
       <c r="F45" s="10" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="G45" s="11" t="inlineStr">
         <is>
-          <t>Steam coal industrial price path, central scenario order of magnitude ~EUR3/GJ</t>
+          <t>Historical and current EUA price context used to anchor the 2025 starting point</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>fuel_prices</t>
+          <t>emission_factors</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>coke</t>
+          <t>coal</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>IPCC</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>World Energy Outlook 2024</t>
+          <t>2006 IPCC Guidelines for National Greenhouse Gas Inventories, Vol. 2 (Energy)</t>
         </is>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/world-energy-outlook-2024</t>
+          <t>https://www.ipcc-nggip.iges.or.jp/public/2006gl/vol2.html</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2006</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>Metallurgical coke priced at a premium to thermal coal (~2x)</t>
+          <t>Default combustion emission factor for coal, ~94 kgCO2/GJ</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="10" t="inlineStr">
         <is>
-          <t>fuel_prices</t>
+          <t>emission_factors</t>
         </is>
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>natural_gas</t>
+          <t>coke</t>
         </is>
       </c>
       <c r="C47" s="10" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>IPCC</t>
         </is>
       </c>
       <c r="D47" s="11" t="inlineStr">
         <is>
-          <t>World Energy Outlook 2024</t>
+          <t>2006 IPCC Guidelines for National Greenhouse Gas Inventories, Vol. 2 (Energy)</t>
         </is>
       </c>
       <c r="E47" s="13" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/world-energy-outlook-2024</t>
+          <t>https://www.ipcc-nggip.iges.or.jp/public/2006gl/vol2.html</t>
         </is>
       </c>
       <c r="F47" s="10" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2006</t>
         </is>
       </c>
       <c r="G47" s="11" t="inlineStr">
         <is>
-          <t>EU industrial natural gas price path, central scenario, declining from ~EUR10/GJ (2025)</t>
+          <t>Default combustion emission factor for coke oven coke, ~107 kgCO2/GJ</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>fuel_prices</t>
+          <t>emission_factors</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>electricity</t>
+          <t>natural_gas</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Eurostat</t>
+          <t>IPCC</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>Electricity price statistics</t>
+          <t>2006 IPCC Guidelines for National Greenhouse Gas Inventories, Vol. 2 (Energy)</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/eurostat/statistics-explained/index.php?title=Electricity_price_statistics</t>
+          <t>https://www.ipcc-nggip.iges.or.jp/public/2006gl/vol2.html</t>
         </is>
       </c>
       <c r="F48" s="6" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2006</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>EU-27 industrial electricity price ~EUR24/GJ (~EUR86/MWh) in 2025, declining as renewables share rises</t>
+          <t>Default combustion emission factor for natural gas, ~56 kgCO2/GJ</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="10" t="inlineStr">
         <is>
-          <t>fuel_prices</t>
+          <t>emission_factors</t>
         </is>
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>hydrogen</t>
+          <t>oil</t>
         </is>
       </c>
       <c r="C49" s="10" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>IPCC</t>
         </is>
       </c>
       <c r="D49" s="11" t="inlineStr">
         <is>
-          <t>Global Hydrogen Review 2024</t>
+          <t>2006 IPCC Guidelines for National Greenhouse Gas Inventories, Vol. 2 (Energy)</t>
         </is>
       </c>
       <c r="E49" s="13" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/global-hydrogen-review-2024</t>
+          <t>https://www.ipcc-nggip.iges.or.jp/public/2006gl/vol2.html</t>
         </is>
       </c>
       <c r="F49" s="10" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2006</t>
         </is>
       </c>
       <c r="G49" s="11" t="inlineStr">
         <is>
-          <t>Low-carbon hydrogen cost path ~EUR40/GJ (~EUR4.8/kg) in 2025 falling to ~EUR20/GJ (~EUR2.4/kg) by 2050</t>
+          <t>Default combustion emission factor for gas/diesel oil &amp; naphtha, ~73 kgCO2/GJ</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>fuel_prices</t>
+          <t>emission_factors</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>biomass</t>
+          <t>hydrogen</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>IEA Bioenergy</t>
+          <t>IPCC AR6 WGIII</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>Decarbonizing industrial process heat: the role of biomass</t>
+          <t>Chapter 11: Industry</t>
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>https://www.ieabioenergy.com/blog/publications/decarbonizing-industrial-process-heat-the-role-of-biomass/</t>
+          <t>https://www.ipcc.ch/report/ar6/wg3/chapter/chapter-11/</t>
         </is>
       </c>
       <c r="F50" s="6" t="inlineStr">
@@ -3030,71 +3047,71 @@
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>Solid biomass/residue fuel price order of magnitude ~EUR8/GJ</t>
+          <t>Zero combustion CO2 for hydrogen; upstream emissions depend on production route (not modelled at combustion stage)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="10" t="inlineStr">
         <is>
-          <t>fuel_prices</t>
+          <t>emission_factors</t>
         </is>
       </c>
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t>oil</t>
+          <t>biomass</t>
         </is>
       </c>
       <c r="C51" s="10" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>IPCC AR6 WGIII</t>
         </is>
       </c>
       <c r="D51" s="11" t="inlineStr">
         <is>
-          <t>World Energy Outlook 2024</t>
+          <t>Chapter 11: Industry</t>
         </is>
       </c>
       <c r="E51" s="13" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/world-energy-outlook-2024</t>
+          <t>https://www.ipcc.ch/report/ar6/wg3/chapter/chapter-11/</t>
         </is>
       </c>
       <c r="F51" s="10" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="G51" s="11" t="inlineStr">
         <is>
-          <t>Industrial oil/naphtha price path, central scenario order of magnitude ~EUR14/GJ</t>
+          <t>Biomass combustion CO2 conventionally reported as zero at point of combustion (biogenic carbon accounting); land-use/supply-chain emissions not modelled here</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>carbon_price</t>
+          <t>emission_factors</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>eu_ets</t>
+          <t>electricity</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>European Commission (DG CLIMA)</t>
+          <t>European Environment Agency (EEA)</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>2040 Climate Target</t>
+          <t>Greenhouse gas emission intensity of electricity generation (indicator)</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>https://commission.europa.eu/topics/climate-action/eu-climate-energy-and-environmental-targets/2040-targets_en</t>
+          <t>https://www.eea.europa.eu/en/analysis/indicators/greenhouse-gas-emission-intensity-of-1</t>
         </is>
       </c>
       <c r="F52" s="6" t="inlineStr">
@@ -3104,404 +3121,404 @@
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>Central EU ETS price path ~EUR80/t (2025) rising to ~EUR200/t (2040) and ~EUR250/t (2050); low/high bands constructed around this by the model team, consistent with the range of EC impact-assessment and market-forward modelling</t>
+          <t>EU-27 grid emission factor ~0.065 tCO2/GJ (~230 gCO2/kWh) in 2025 falling to ~0.003 tCO2/GJ by 2050 as the grid decarbonises</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="10" t="inlineStr">
         <is>
-          <t>carbon_price</t>
+          <t>constraints</t>
         </is>
       </c>
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t>eu_ets</t>
+          <t>scrap_share_max</t>
         </is>
       </c>
       <c r="C53" s="10" t="inlineStr">
         <is>
-          <t>ICAP</t>
+          <t>Material Economics</t>
         </is>
       </c>
       <c r="D53" s="11" t="inlineStr">
         <is>
-          <t>EU Emissions Trading System (EU ETS)</t>
+          <t>Industrial Transformation 2050 - Pathways to Net-Zero Emissions from EU Heavy Industry</t>
         </is>
       </c>
       <c r="E53" s="13" t="inlineStr">
         <is>
-          <t>https://icapcarbonaction.com/en/ets/eu-emissions-trading-system-eu-ets</t>
+          <t>https://materialeconomics.com/sites/default/files/2024-06/material-economics-industrial-transformation-2050-executive-summary.pdf</t>
         </is>
       </c>
       <c r="F53" s="10" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="G53" s="11" t="inlineStr">
         <is>
-          <t>Historical and current EUA price context used to anchor the 2025 starting point</t>
+          <t>Steel scrap availability rising from ~45% (2025) to ~55% (2050) of demand servable by scrap-EAF; aluminium secondary share rising ~55% to ~65%, both circularity-constrained</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>emission_factors</t>
+          <t>constraints</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>coal</t>
+          <t>biomass_pj_max</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>IPCC</t>
+          <t>JRC (European Commission)</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>2006 IPCC Guidelines for National Greenhouse Gas Inventories, Vol. 2 (Energy)</t>
+          <t>Brief on biomass for energy in the European Union</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>https://www.ipcc-nggip.iges.or.jp/public/2006gl/vol2.html</t>
+          <t>https://publications.jrc.ec.europa.eu/repository/handle/JRC109354</t>
         </is>
       </c>
       <c r="F54" s="6" t="inlineStr">
         <is>
-          <t>2006</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="G54" s="7" t="inlineStr">
         <is>
-          <t>Default combustion emission factor for coal, ~94 kgCO2/GJ</t>
+          <t>Sustainable biomass availability for industrial energy use constrained to an order-of-magnitude ceiling of ~300 PJ/yr across all EU-27 industry</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>emission_factors</t>
+          <t>constraints</t>
         </is>
       </c>
       <c r="B55" s="10" t="inlineStr">
         <is>
-          <t>coke</t>
+          <t>ccs_mt_max</t>
         </is>
       </c>
       <c r="C55" s="10" t="inlineStr">
         <is>
-          <t>IPCC</t>
+          <t>Global CCS Institute</t>
         </is>
       </c>
       <c r="D55" s="11" t="inlineStr">
         <is>
-          <t>2006 IPCC Guidelines for National Greenhouse Gas Inventories, Vol. 2 (Energy)</t>
+          <t>Global Status of CCS report series</t>
         </is>
       </c>
       <c r="E55" s="13" t="inlineStr">
         <is>
-          <t>https://www.ipcc-nggip.iges.or.jp/public/2006gl/vol2.html</t>
+          <t>https://www.globalccsinstitute.com/</t>
         </is>
       </c>
       <c r="F55" s="10" t="inlineStr">
         <is>
-          <t>2006</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="G55" s="11" t="inlineStr">
         <is>
-          <t>Default combustion emission factor for coke oven coke, ~107 kgCO2/GJ</t>
+          <t>EU CO2 transport &amp; storage network ramp-up: ~0 Mt/yr (2025) to ~100 Mt/yr (2050) capturable across all subsectors</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>emission_factors</t>
+          <t>constraints</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>natural_gas</t>
+          <t>ccs_mt_max</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>IPCC</t>
+          <t>Clean Air Task Force</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>2006 IPCC Guidelines for National Greenhouse Gas Inventories, Vol. 2 (Energy)</t>
+          <t>Carbon capture and storage in Europe: slow but significant progress in 2025</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>https://www.ipcc-nggip.iges.or.jp/public/2006gl/vol2.html</t>
+          <t>https://www.catf.us/2025/11/carbon-capture-storage-europe-slow-but-significant-progress-2025/</t>
         </is>
       </c>
       <c r="F56" s="6" t="inlineStr">
         <is>
-          <t>2006</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>Default combustion emission factor for natural gas, ~56 kgCO2/GJ</t>
+          <t>Status of first EU CO2 storage/transport projects (Northern Lights, Porthos, Greensand) calibrating the near-term ramp</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="10" t="inlineStr">
         <is>
-          <t>emission_factors</t>
+          <t>demand</t>
         </is>
       </c>
       <c r="B57" s="10" t="inlineStr">
         <is>
-          <t>oil</t>
+          <t>steel</t>
         </is>
       </c>
       <c r="C57" s="10" t="inlineStr">
         <is>
-          <t>IPCC</t>
+          <t>Eurofer</t>
         </is>
       </c>
       <c r="D57" s="11" t="inlineStr">
         <is>
-          <t>2006 IPCC Guidelines for National Greenhouse Gas Inventories, Vol. 2 (Energy)</t>
+          <t>European Steel in Figures 2024</t>
         </is>
       </c>
       <c r="E57" s="13" t="inlineStr">
         <is>
-          <t>https://www.ipcc-nggip.iges.or.jp/public/2006gl/vol2.html</t>
+          <t>https://www.eurofer.eu/publications/brochures-booklets-and-factsheets/european-steel-in-figures-2024</t>
         </is>
       </c>
       <c r="F57" s="10" t="inlineStr">
         <is>
-          <t>2006</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="G57" s="11" t="inlineStr">
         <is>
-          <t>Default combustion emission factor for gas/diesel oil &amp; naphtha, ~73 kgCO2/GJ</t>
+          <t>Demand path assumed broadly flat-to-declining from the 2023 production base</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>emission_factors</t>
+          <t>demand</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>hydrogen</t>
+          <t>cement</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>IPCC AR6 WGIII</t>
+          <t>Cembureau</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>Chapter 11: Industry</t>
+          <t>Key Facts &amp; Figures</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>https://www.ipcc.ch/report/ar6/wg3/chapter/chapter-11/</t>
+          <t>https://www.cembureau.eu/media/00ejjcfj/key-facts-figures-publication-june-2024.pdf</t>
         </is>
       </c>
       <c r="F58" s="6" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>Zero combustion CO2 for hydrogen; upstream emissions depend on production route (not modelled at combustion stage)</t>
+          <t>Demand path assumed broadly flat-to-declining from the 2023 production base</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="10" t="inlineStr">
         <is>
-          <t>emission_factors</t>
+          <t>demand</t>
         </is>
       </c>
       <c r="B59" s="10" t="inlineStr">
         <is>
-          <t>biomass</t>
+          <t>aluminium</t>
         </is>
       </c>
       <c r="C59" s="10" t="inlineStr">
         <is>
-          <t>IPCC AR6 WGIII</t>
+          <t>International Aluminium Institute (IAI)</t>
         </is>
       </c>
       <c r="D59" s="11" t="inlineStr">
         <is>
-          <t>Chapter 11: Industry</t>
+          <t>Statistics</t>
         </is>
       </c>
       <c r="E59" s="13" t="inlineStr">
         <is>
-          <t>https://www.ipcc.ch/report/ar6/wg3/chapter/chapter-11/</t>
+          <t>https://international-aluminium.org/statistics/</t>
         </is>
       </c>
       <c r="F59" s="10" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="G59" s="11" t="inlineStr">
         <is>
-          <t>Biomass combustion CO2 conventionally reported as zero at point of combustion (biogenic carbon accounting); land-use/supply-chain emissions not modelled here</t>
+          <t>Demand path assumed slight growth, reflecting continued electrification-driven aluminium demand</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>emission_factors</t>
+          <t>demand</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>electricity</t>
+          <t>hvc</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>European Environment Agency (EEA)</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>Greenhouse gas emission intensity of electricity generation (indicator)</t>
+          <t>The Future of Petrochemicals</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>https://www.eea.europa.eu/en/analysis/indicators/greenhouse-gas-emission-intensity-of-1</t>
+          <t>https://www.iea.org/reports/the-future-of-petrochemicals</t>
         </is>
       </c>
       <c r="F60" s="6" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2018</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>EU-27 grid emission factor ~0.065 tCO2/GJ (~230 gCO2/kWh) in 2025 falling to ~0.003 tCO2/GJ by 2050 as the grid decarbonises</t>
+          <t>Demand path assumed slight growth</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="10" t="inlineStr">
         <is>
-          <t>constraints</t>
+          <t>technologies</t>
         </is>
       </c>
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t>scrap_share_max</t>
+          <t>discount_rate</t>
         </is>
       </c>
       <c r="C61" s="10" t="inlineStr">
         <is>
-          <t>Material Economics</t>
+          <t>IPCC</t>
         </is>
       </c>
       <c r="D61" s="11" t="inlineStr">
         <is>
-          <t>Industrial Transformation 2050 - Pathways to Net-Zero Emissions from EU Heavy Industry</t>
+          <t>AR6 WGIII, Chapter 11: Industry</t>
         </is>
       </c>
       <c r="E61" s="13" t="inlineStr">
         <is>
-          <t>https://materialeconomics.com/sites/default/files/2024-06/material-economics-industrial-transformation-2050-executive-summary.pdf</t>
+          <t>https://www.ipcc.ch/report/ar6/wg3/chapter/chapter-11/</t>
         </is>
       </c>
       <c r="F61" s="10" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="G61" s="11" t="inlineStr">
         <is>
-          <t>Steel scrap availability rising from ~45% (2025) to ~55% (2050) of demand servable by scrap-EAF; aluminium secondary share rising ~55% to ~65%, both circularity-constrained</t>
+          <t>7% social/industry discount rate and capital recovery factor approach used to annualise CAPEX, consistent with standard industrial decarbonisation cost-modelling practice</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>constraints</t>
+          <t>demand</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>biomass_pj_max</t>
+          <t>ammonia</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>JRC (European Commission)</t>
+          <t>Fertilizers Europe</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>Brief on biomass for energy in the European Union</t>
+          <t>Fertilizer Industry Facts and Figures 2023 edition</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>https://publications.jrc.ec.europa.eu/repository/handle/JRC109354</t>
+          <t>https://www.fertilizerseurope.com/publications/fertilizers-industry-facts-and-figures-2023-edition/</t>
         </is>
       </c>
       <c r="F62" s="6" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>Sustainable biomass availability for industrial energy use constrained to an order-of-magnitude ceiling of ~300 PJ/yr across all EU-27 industry</t>
+          <t>Demand path assumed broadly flat-to-slightly-declining from the 2023 production base</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="10" t="inlineStr">
         <is>
-          <t>constraints</t>
+          <t>demand</t>
         </is>
       </c>
       <c r="B63" s="10" t="inlineStr">
         <is>
-          <t>ccs_mt_max</t>
+          <t>glass</t>
         </is>
       </c>
       <c r="C63" s="10" t="inlineStr">
         <is>
-          <t>Global CCS Institute</t>
+          <t>FEVE (European Container Glass Federation)</t>
         </is>
       </c>
       <c r="D63" s="11" t="inlineStr">
         <is>
-          <t>Global Status of CCS report series</t>
+          <t>Statistics</t>
         </is>
       </c>
       <c r="E63" s="13" t="inlineStr">
         <is>
-          <t>https://www.globalccsinstitute.com/</t>
+          <t>https://feve.org/about-glass/statistics/</t>
         </is>
       </c>
       <c r="F63" s="10" t="inlineStr">
@@ -3511,108 +3528,108 @@
       </c>
       <c r="G63" s="11" t="inlineStr">
         <is>
-          <t>EU CO2 transport &amp; storage network ramp-up: ~0 Mt/yr (2025) to ~100 Mt/yr (2050) capturable across all subsectors</t>
+          <t>Demand path assumed broadly flat from the 2023 production base</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>constraints</t>
+          <t>demand</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>ccs_mt_max</t>
+          <t>paper</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>Clean Air Task Force</t>
+          <t>CEPI</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>Carbon capture and storage in Europe: slow but significant progress in 2025</t>
+          <t>Key Statistics 2022 - European pulp &amp; paper industry</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>https://www.catf.us/2025/11/carbon-capture-storage-europe-slow-but-significant-progress-2025/</t>
+          <t>https://www.cepi.org/wp-content/uploads/2023/07/2022-Key-Statistics-FINAL.pdf</t>
         </is>
       </c>
       <c r="F64" s="6" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>Status of first EU CO2 storage/transport projects (Northern Lights, Porthos, Greensand) calibrating the near-term ramp</t>
+          <t>Demand path assumed gently declining from the 2023 production base</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="10" t="inlineStr">
         <is>
-          <t>demand</t>
+          <t>scenarios</t>
         </is>
       </c>
       <c r="B65" s="10" t="inlineStr">
         <is>
-          <t>steel</t>
+          <t>multiple</t>
         </is>
       </c>
       <c r="C65" s="10" t="inlineStr">
         <is>
-          <t>Eurofer</t>
+          <t>ESABCC Method Hub (model team)</t>
         </is>
       </c>
       <c r="D65" s="11" t="inlineStr">
         <is>
-          <t>European Steel in Figures 2024</t>
-        </is>
-      </c>
-      <c r="E65" s="13" t="inlineStr">
-        <is>
-          <t>https://www.eurofer.eu/publications/brochures-booklets-and-factsheets/european-steel-in-figures-2024</t>
+          <t>Model README - sensitivity scenario methodology</t>
+        </is>
+      </c>
+      <c r="E65" s="11" t="inlineStr">
+        <is>
+          <t>beta/modules/summer-prep/optimization/model/README.md</t>
         </is>
       </c>
       <c r="F65" s="10" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="G65" s="11" t="inlineStr">
         <is>
-          <t>Demand path assumed broadly flat-to-declining from the 2023 production base</t>
+          <t>All 13 scenarios (1 central + 12 sensitivities) are prototype modelling assumptions (parameter multipliers applied to already-sourced central inputs), not independent literature values; see the README for the full methodology and per-scenario definitions.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>demand</t>
+          <t>technologies</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>cement</t>
+          <t>steel_bfbof_ccs</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>Cembureau</t>
+          <t>Danish Energy Agency</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>Key Facts &amp; Figures</t>
+          <t>Technology Data for Carbon Capture, Transport and Storage</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>https://www.cembureau.eu/media/00ejjcfj/key-facts-figures-publication-june-2024.pdf</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-carbon-capture-transport-and-storage</t>
         </is>
       </c>
       <c r="F66" s="6" t="inlineStr">
@@ -3622,34 +3639,34 @@
       </c>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>Demand path assumed broadly flat-to-declining from the 2023 production base</t>
+          <t>Sheet 401.c (post-combustion capture, cement-kiln flue gas, used as CO2-concentration proxy for BF-BOF top gas): specific investment, fixed/var O&amp;M per tCO2 captured, 25-yr capture-unit lifetime; now the primary source, replacing the generic IEAGHG (2018) estimate.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="10" t="inlineStr">
         <is>
-          <t>demand</t>
+          <t>technologies</t>
         </is>
       </c>
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t>aluminium</t>
+          <t>cement_ccs</t>
         </is>
       </c>
       <c r="C67" s="10" t="inlineStr">
         <is>
-          <t>International Aluminium Institute (IAI)</t>
+          <t>Danish Energy Agency</t>
         </is>
       </c>
       <c r="D67" s="11" t="inlineStr">
         <is>
-          <t>Statistics</t>
+          <t>Technology Data for Carbon Capture, Transport and Storage</t>
         </is>
       </c>
       <c r="E67" s="13" t="inlineStr">
         <is>
-          <t>https://international-aluminium.org/statistics/</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-carbon-capture-transport-and-storage</t>
         </is>
       </c>
       <c r="F67" s="10" t="inlineStr">
@@ -3659,44 +3676,44 @@
       </c>
       <c r="G67" s="11" t="inlineStr">
         <is>
-          <t>Demand path assumed slight growth, reflecting continued electrification-driven aluminium demand</t>
+          <t>Sheet 401.c (post-combustion capture retrofit, 4500 t clinker/day cement kiln - a direct technology match): specific investment, fixed/var O&amp;M per tCO2 captured, 25-yr capture-unit lifetime; now the primary source, replacing the generic IEAGHG (2018) estimate. Heidelberg Materials retained for available_from calibration.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>demand</t>
+          <t>technologies</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>hvc</t>
+          <t>cement_altfuel</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>Danish Energy Agency</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>The Future of Petrochemicals</t>
+          <t>Technology Data for Industrial Process Heat</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/the-future-of-petrochemicals</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-industrial-process-heat</t>
         </is>
       </c>
       <c r="F68" s="6" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>Demand path assumed slight growth</t>
+          <t>Sheet 7.2 (direct firing of solid fuels, 100% net efficiency) used as the closest available DEA proxy for alternative/biomass kiln-fuel firing; DEA has no cement-kiln-specific alt-fuel sheet, so IEA/CSI (2018) is retained for kiln-level capex/opex/lifetime, with DEA as the primary technical cross-check per the model's DEA-primary-source policy.</t>
         </is>
       </c>
     </row>
@@ -3708,59 +3725,59 @@
       </c>
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t>discount_rate</t>
+          <t>hvc_elec</t>
         </is>
       </c>
       <c r="C69" s="10" t="inlineStr">
         <is>
-          <t>IPCC</t>
+          <t>Danish Energy Agency</t>
         </is>
       </c>
       <c r="D69" s="11" t="inlineStr">
         <is>
-          <t>AR6 WGIII, Chapter 11: Industry</t>
+          <t>Technology Data for Industrial Process Heat</t>
         </is>
       </c>
       <c r="E69" s="13" t="inlineStr">
         <is>
-          <t>https://www.ipcc.ch/report/ar6/wg3/chapter/chapter-11/</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-industrial-process-heat</t>
         </is>
       </c>
       <c r="F69" s="10" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="G69" s="11" t="inlineStr">
         <is>
-          <t>7% social/industry discount rate and capital recovery factor approach used to annualise CAPEX, consistent with standard industrial decarbonisation cost-modelling practice</t>
+          <t>Sheet 7.3 (direct electric firing, 100% net efficiency, up to 2000 degC) confirms electrified cracking-furnace heat supply is well within DEA's technical envelope; DEA prices heating elements only, so BASF/SABIC/Linde (2024) is retained for full e-cracker capex/opex/lifetime, with DEA as the primary technical cross-check per the model's DEA-primary-source policy.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>demand</t>
+          <t>technologies</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>ammonia</t>
+          <t>hvc_ccs</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>Fertilizers Europe</t>
+          <t>Danish Energy Agency</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>Fertilizer Industry Facts and Figures 2023 edition</t>
+          <t>Technology Data for Carbon Capture, Transport and Storage</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>https://www.fertilizerseurope.com/publications/fertilizers-industry-facts-and-figures-2023-edition/</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-carbon-capture-transport-and-storage</t>
         </is>
       </c>
       <c r="F70" s="6" t="inlineStr">
@@ -3770,34 +3787,34 @@
       </c>
       <c r="G70" s="7" t="inlineStr">
         <is>
-          <t>Demand path assumed broadly flat-to-slightly-declining from the 2023 production base</t>
+          <t>Sheet 401.a (post-combustion capture, dilute ~15% CO2 CHP/biomass flue gas, used as proxy for cracker-furnace flue gas - DEA has no HVC-specific sheet): specific investment, fixed/var O&amp;M per tCO2 captured, 25-yr capture-unit lifetime; now the primary source, replacing the generic IEAGHG (2018) estimate.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="10" t="inlineStr">
         <is>
-          <t>demand</t>
+          <t>technologies</t>
         </is>
       </c>
       <c r="B71" s="10" t="inlineStr">
         <is>
-          <t>glass</t>
+          <t>ammonia_smr_ccs</t>
         </is>
       </c>
       <c r="C71" s="10" t="inlineStr">
         <is>
-          <t>FEVE (European Container Glass Federation)</t>
+          <t>Danish Energy Agency</t>
         </is>
       </c>
       <c r="D71" s="11" t="inlineStr">
         <is>
-          <t>Statistics</t>
+          <t>Technology Data for Carbon Capture, Transport and Storage</t>
         </is>
       </c>
       <c r="E71" s="13" t="inlineStr">
         <is>
-          <t>https://feve.org/about-glass/statistics/</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-carbon-capture-transport-and-storage</t>
         </is>
       </c>
       <c r="F71" s="10" t="inlineStr">
@@ -3807,86 +3824,345 @@
       </c>
       <c r="G71" s="11" t="inlineStr">
         <is>
-          <t>Demand path assumed broadly flat from the 2023 production base</t>
+          <t>Sheet 401.c (post-combustion capture, cement-kiln flue gas used as moderate-CO2-concentration proxy - DEA has no SMR/ammonia-specific sheet): specific investment, fixed/var O&amp;M per tCO2 captured, 25-yr capture-unit lifetime; now the primary source, replacing the IEA (2021) Ammonia Technology Roadmap-implied capture premium.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>demand</t>
+          <t>technologies</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>paper</t>
+          <t>ammonia_h2</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>CEPI</t>
+          <t>Danish Energy Agency</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>Key Statistics 2022 - European pulp &amp; paper industry</t>
+          <t>Technology Data for Renewable Fuels</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>https://www.cepi.org/wp-content/uploads/2023/07/2022-Key-Statistics-FINAL.pdf</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-renewable-fuels</t>
         </is>
       </c>
       <c r="F72" s="6" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>Demand path assumed gently declining from the 2023 production base</t>
+          <t>Sheet 5.4 (Hydrogen to Ammonia, Haber-Bosch synthesis excl. electrolyser and excl. ASU): specific investment, fixed/var O&amp;M, 30-yr lifetime; now the primary source. Correctly excludes electrolyser capex, which is already reflected in the purchased-hydrogen carrier price (see fuel_prices,hydrogen below), avoiding the double-counting implicit in the prior IEA (2021) Ammonia Technology Roadmap Executive Summary bundled estimate. Yara International (2024) retained for available_from calibration.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="10" t="inlineStr">
         <is>
-          <t>scenarios</t>
+          <t>technologies</t>
         </is>
       </c>
       <c r="B73" s="10" t="inlineStr">
         <is>
+          <t>glass_elec</t>
+        </is>
+      </c>
+      <c r="C73" s="10" t="inlineStr">
+        <is>
+          <t>Danish Energy Agency</t>
+        </is>
+      </c>
+      <c r="D73" s="11" t="inlineStr">
+        <is>
+          <t>Technology Data for Industrial Process Heat</t>
+        </is>
+      </c>
+      <c r="E73" s="13" t="inlineStr">
+        <is>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-industrial-process-heat</t>
+        </is>
+      </c>
+      <c r="F73" s="10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G73" s="11" t="inlineStr">
+        <is>
+          <t>Sheet 7.3 (direct electric firing: 100% net efficiency, up to 2000 degC, 20-yr technical lifetime) confirms all-electric glass melting is well within DEA's technical envelope and grounds the updated 20-yr lifetime; DEA prices heating elements only (not furnace shell/refractories/forming equipment), so IEA (2024) ETP is retained for furnace-level capex/opex, with DEA as the primary technical cross-check per the model's DEA-primary-source policy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>technologies</t>
+        </is>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>glass_hybrid</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>Danish Energy Agency</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="inlineStr">
+        <is>
+          <t>Technology Data for Industrial Process Heat</t>
+        </is>
+      </c>
+      <c r="E74" s="9" t="inlineStr">
+        <is>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-industrial-process-heat</t>
+        </is>
+      </c>
+      <c r="F74" s="6" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G74" s="7" t="inlineStr">
+        <is>
+          <t>Blend of sheet 7.3 (direct electric firing) and sheet 6.1 (gas/oil boiler) as proxies for the electric and gas-fired shares of a hybrid furnace; grounds the updated 18-yr lifetime. DEA prices heating elements/burners only, so IEA (2024) ETP is retained for furnace-level capex/opex, with DEA as the primary technical cross-check per the model's DEA-primary-source policy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="10" t="inlineStr">
+        <is>
+          <t>technologies</t>
+        </is>
+      </c>
+      <c r="B75" s="10" t="inlineStr">
+        <is>
+          <t>paper_elec</t>
+        </is>
+      </c>
+      <c r="C75" s="10" t="inlineStr">
+        <is>
+          <t>Danish Energy Agency</t>
+        </is>
+      </c>
+      <c r="D75" s="11" t="inlineStr">
+        <is>
+          <t>Technology Data for Industrial Process Heat</t>
+        </is>
+      </c>
+      <c r="E75" s="13" t="inlineStr">
+        <is>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-industrial-process-heat</t>
+        </is>
+      </c>
+      <c r="F75" s="10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G75" s="11" t="inlineStr">
+        <is>
+          <t>Sheet 2.a (high-temperature heat pump up to 125 degC): COP 2.7-2.95 (2025-2050), 1.15 M EUR/MW nominal investment (2030 est.), 20-yr technical lifetime; now the primary source, replacing IEA (2022) Future of Heat Pumps as the quantitative basis for capex, electricity intensity and lifetime.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>technologies</t>
+        </is>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>paper_bio</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>Danish Energy Agency</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="inlineStr">
+        <is>
+          <t>Technology Data for Industrial Process Heat</t>
+        </is>
+      </c>
+      <c r="E76" s="9" t="inlineStr">
+        <is>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-industrial-process-heat</t>
+        </is>
+      </c>
+      <c r="F76" s="6" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G76" s="7" t="inlineStr">
+        <is>
+          <t>Sheet 6.2 (biomass boiler): 88.9% annual-average efficiency, 0.878 M EUR/MW nominal investment (2025), 25-yr technical lifetime; now the primary source, replacing IEA Bioenergy (2022) as the quantitative basis for capex, fuel intensity and lifetime.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="10" t="inlineStr">
+        <is>
+          <t>fuel_prices</t>
+        </is>
+      </c>
+      <c r="B77" s="10" t="inlineStr">
+        <is>
+          <t>hydrogen</t>
+        </is>
+      </c>
+      <c r="C77" s="10" t="inlineStr">
+        <is>
+          <t>Danish Energy Agency</t>
+        </is>
+      </c>
+      <c r="D77" s="11" t="inlineStr">
+        <is>
+          <t>Technology Data for Renewable Fuels</t>
+        </is>
+      </c>
+      <c r="E77" s="13" t="inlineStr">
+        <is>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-renewable-fuels</t>
+        </is>
+      </c>
+      <c r="F77" s="10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G77" s="11" t="inlineStr">
+        <is>
+          <t>Sheet 1.1 (alkaline electrolysis, AEC, 100 MW plant): bottom-up levelised cost of hydrogen from DEA electrolyser capex (975-&gt;300 EUR/kW, 2025-&gt;2050), 4%/yr fixed O&amp;M, 25-yr lifetime (7% WACC CRF), DEA stack+BOP electricity consumption (56.7-&gt;47.6 kWh/kg H2), 8000 full-load h/yr, and this model's own Eurostat electricity price path; now the primary source, replacing the IEA (2024) Global Hydrogen Review market-price path, which this bottom-up calculation shows was materially more optimistic (17-40% below the DEA-grounded figure, widening over the horizon).</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="inlineStr">
+        <is>
+          <t>fuel_prices</t>
+        </is>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>electricity</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="inlineStr">
+        <is>
+          <t>Danish Energy Agency</t>
+        </is>
+      </c>
+      <c r="D78" s="7" t="inlineStr">
+        <is>
+          <t>Technology Data for Generation of Electricity and District Heat</t>
+        </is>
+      </c>
+      <c r="E78" s="9" t="inlineStr">
+        <is>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-generation-electricity-and-district-heating</t>
+        </is>
+      </c>
+      <c r="F78" s="6" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G78" s="7" t="inlineStr">
+        <is>
+          <t>Reviewed as a possible source for the industrial electricity price path but not adopted: this DEA catalogue prices generation technologies (LCOE), not the retail/industrial electricity price this table needs, so Eurostat market-price statistics remain the more appropriate and directly applicable source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="10" t="inlineStr">
+        <is>
+          <t>fuel_prices</t>
+        </is>
+      </c>
+      <c r="B79" s="10" t="inlineStr">
+        <is>
+          <t>biomass</t>
+        </is>
+      </c>
+      <c r="C79" s="10" t="inlineStr">
+        <is>
+          <t>Danish Energy Agency</t>
+        </is>
+      </c>
+      <c r="D79" s="11" t="inlineStr">
+        <is>
+          <t>Technology Data for Renewable Fuels</t>
+        </is>
+      </c>
+      <c r="E79" s="13" t="inlineStr">
+        <is>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-renewable-fuels</t>
+        </is>
+      </c>
+      <c r="F79" s="10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="G79" s="11" t="inlineStr">
+        <is>
+          <t>Reviewed as a possible source for the biomass feedstock price path but not adopted: this DEA catalogue prices biomass-conversion plant technologies (boilers, gasifiers, pyrolysis), not EU biomass feedstock market prices, so the IEA Bioenergy feedstock-price estimate is retained.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="inlineStr">
+        <is>
+          <t>technologies</t>
+        </is>
+      </c>
+      <c r="B80" s="6" t="inlineStr">
+        <is>
           <t>multiple</t>
         </is>
       </c>
-      <c r="C73" s="10" t="inlineStr">
-        <is>
-          <t>ESABCC Method Hub (model team)</t>
-        </is>
-      </c>
-      <c r="D73" s="11" t="inlineStr">
-        <is>
-          <t>Model README - sensitivity scenario methodology</t>
-        </is>
-      </c>
-      <c r="E73" s="11" t="inlineStr">
-        <is>
-          <t>beta/modules/summer-prep/optimization/model/README.md</t>
-        </is>
-      </c>
-      <c r="F73" s="10" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="G73" s="11" t="inlineStr">
-        <is>
-          <t>All 13 scenarios (1 central + 12 sensitivities) are prototype modelling assumptions (parameter multipliers applied to already-sourced central inputs), not independent literature values; see the README for the full methodology and per-scenario definitions.</t>
+      <c r="C80" s="6" t="inlineStr">
+        <is>
+          <t>Danish Energy Agency</t>
+        </is>
+      </c>
+      <c r="D80" s="7" t="inlineStr">
+        <is>
+          <t>Technology Data catalogue series (Industrial Process Heat; Carbon Capture, Transport and Storage; Renewable Fuels; Generation of Electricity and District Heat)</t>
+        </is>
+      </c>
+      <c r="E80" s="9" t="inlineStr">
+        <is>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data</t>
+        </is>
+      </c>
+      <c r="F80" s="6" t="inlineStr">
+        <is>
+          <t>2024-2026</t>
+        </is>
+      </c>
+      <c r="G80" s="7" t="inlineStr">
+        <is>
+          <t>Per explicit user direction, the DEA Technology Data catalogue series is the primary source for this model wherever it plausibly covers the underlying equipment (all CCS variants; paper/glass/HVC electrification and biomass/alt-fuel heat; electrolytic-hydrogen ammonia synthesis and the hydrogen price path). Where DEA genuinely has no coverage (BF-BOF/DRI/EAF steel process metallurgy, cement clinker kilns, steam crackers, aluminium smelting, SMR reforming), the pre-existing IEA/IEAGHG/JRC/etc. sources remain primary - DEA is primary, not exclusive, consistent with data-quality requirements.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G73"/>
+  <autoFilter ref="A1:G80"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
@@ -3951,14 +4227,21 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E75" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E76" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="rId78"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5483,13 +5766,13 @@
         </is>
       </c>
       <c r="D3" s="19" t="n">
-        <v>650</v>
+        <v>770</v>
       </c>
       <c r="E3" s="19" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F3" s="19" t="n">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="G3" s="15" t="n">
         <v>25</v>
@@ -5508,12 +5791,12 @@
       </c>
       <c r="L3" s="11" t="inlineStr">
         <is>
-          <t>IEAGHG (2018), Cost of CO2 capture in the industrial sector: cement and iron &amp; steel industries (2018-TR03)</t>
+          <t>Danish Energy Agency (2024), Technology Data for Carbon Capture, Transport and Storage (sheet 401.c, post-combustion capture retrofit, cement kiln flue gas used as CO2-concentration proxy for BF-BOF flue/top gas, ~90% capture); converted at 1.185 tCO2 captured/t steel (combustion CO2 at 0.6 capture rate), 8000 full-load h/yr, DEA specific investment 2.5 M EUR/(tCO2/h) (2030) -&gt; capture add-on 370 EUR/(t/yr) added to unchanged base steel_bfbof capex (400); base process still IEA (2020) Iron and Steel Technology Roadmap. DEA capture-retrofit benchmark implies a materially higher capture add-on than the prior generic IEAGHG (2018) estimate (250 EUR/t) - adopted the DEA-grounded (higher, more conservative) figure and retained it for fixed/var O&amp;M add-ons (11.9 and 3.0 EUR/t respectively, close to the prior estimate).</t>
         </is>
       </c>
       <c r="M3" s="13" t="inlineStr">
         <is>
-          <t>https://ieaghg.org/publications/cost-of-co2-capture-in-the-industrial-sector-cement-and-iron-and-steel-industries/</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-carbon-capture-transport-and-storage</t>
         </is>
       </c>
     </row>
@@ -5789,16 +6072,16 @@
         </is>
       </c>
       <c r="D9" s="19" t="n">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="E9" s="19" t="n">
+        <v>18</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>26</v>
+      </c>
+      <c r="G9" s="15" t="n">
         <v>25</v>
-      </c>
-      <c r="F9" s="19" t="n">
-        <v>35</v>
-      </c>
-      <c r="G9" s="15" t="n">
-        <v>30</v>
       </c>
       <c r="H9" s="15" t="n">
         <v>2028</v>
@@ -5814,12 +6097,12 @@
       </c>
       <c r="L9" s="11" t="inlineStr">
         <is>
-          <t>IEAGHG (2018), Cost of CO2 capture in the industrial sector: cement and iron &amp; steel industries (2018-TR03); Heidelberg Materials (2025), World premiere: CCS cement facility opens in Norway (Brevik CCS)</t>
+          <t>Danish Energy Agency (2024), Technology Data for Carbon Capture, Transport and Storage (sheet 401.c, post-combustion capture retrofit for a 4500 t clinker/day cement kiln - a direct match for this technology); converted at 0.567 tCO2 captured/t clinker (0.9 capture rate on ~0.63 tCO2/t pre-capture process+combustion CO2), 8000 full-load h/yr, DEA specific investment 2.5 M EUR/(tCO2/h) (2030) -&gt; capture add-on ~177 EUR/(t/yr) on top of the unchanged cement_ref kiln capex (150), materially consistent with the prior implied add-on (170 EUR/t from IEAGHG 2018); fixed/var O&amp;M add-ons recomputed from DEA (5.7 and 1.4 EUR/t) and are lower than the prior generic IEAGHG estimate - adopted the DEA, more granular, figures. Capture-unit lifetime (25 yr per DEA) now governs over the kiln's own 35-yr structural life, since capture equipment would need reinvestment first. Heidelberg Materials (2025) Brevik CCS start-up retained for the available_from=2028 calibration.</t>
         </is>
       </c>
       <c r="M9" s="13" t="inlineStr">
         <is>
-          <t>https://ieaghg.org/publications/cost-of-co2-capture-in-the-industrial-sector-cement-and-iron-and-steel-industries/</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-carbon-capture-transport-and-storage</t>
         </is>
       </c>
     </row>
@@ -5865,12 +6148,12 @@
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
-          <t>IEA / CSI (2018), Technology Roadmap: Low-Carbon Transition in the Cement Industry</t>
+          <t>Danish Energy Agency (2026), Technology Data for Industrial Process Heat (sheet 7.2, direct firing of solid fuels: 100% net efficiency, used as the closest available DEA proxy for alternative/biomass fuel firing in a cement kiln burner - DEA has no cement-kiln-specific alt-fuel sheet). Capex/fixed/var opex and the 35-yr lifetime retained from IEA / CSI (2018) Technology Roadmap: Low-Carbon Transition in the Cement Industry: DEA's burner-only figures (0.258 M EUR/MW, 15-yr burner lifetime) price the firing equipment alone, not the rotary kiln shell/refractories/preheater that dominate cement-kiln capex and govern its much longer structural life - divergence noted, fuller-scope IEA/CSI figures kept.</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/technology-roadmap-low-carbon-transition-in-the-cement-industry</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-industrial-process-heat</t>
         </is>
       </c>
     </row>
@@ -5967,12 +6250,12 @@
       </c>
       <c r="L12" s="7" t="inlineStr">
         <is>
-          <t>BASF / SABIC / Linde (2024), Start-up of the world's first large-scale electrically heated steam cracking furnace</t>
+          <t>Danish Energy Agency (2026), Technology Data for Industrial Process Heat (sheet 7.3, direct electric firing: 100% net efficiency, heat supply up to 2000 degC, technically consistent with electrically heated cracking-furnace tube temperatures ~850 degC). Capex/fixed/var opex and the 30-yr lifetime retained from BASF / SABIC / Linde (2024)'s e-cracker demonstration: DEA's sheet prices resistive heating elements alone (~0.07 M EUR/MW, converting to a small fraction of this technology's capex) and excludes the cracker tubes, compressors and separation train that dominate real e-cracker capex - a wide divergence, noted, with the fuller-scope BASF-anchored literature figure kept as the defensible capex/opex/lifetime.</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>https://www.basf.com/global/en/media/news-releases/2024/04/p-24-177</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-industrial-process-heat</t>
         </is>
       </c>
     </row>
@@ -6044,16 +6327,16 @@
         </is>
       </c>
       <c r="D14" s="16" t="n">
-        <v>900</v>
+        <v>1020</v>
       </c>
       <c r="E14" s="16" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="F14" s="16" t="n">
-        <v>560</v>
+        <v>555</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="H14" s="14" t="n">
         <v>2032</v>
@@ -6069,12 +6352,12 @@
       </c>
       <c r="L14" s="7" t="inlineStr">
         <is>
-          <t>IEAGHG (2018), Cost of CO2 capture in the industrial sector: cement and iron &amp; steel industries (2018-TR03)</t>
+          <t>Danish Energy Agency (2024), Technology Data for Carbon Capture, Transport and Storage (sheet 401.a, post-combustion capture retrofit on a dilute ~15% CO2 CHP/biomass flue gas, used as the closest available DEA proxy for cracker-furnace flue gas - DEA has no HVC/steam-cracker-specific capture sheet); converted at 0.539 tCO2 captured/t HVC (0.65 capture rate on ~0.83 tCO2/t pre-capture combustion CO2), 8000 full-load h/yr, DEA specific investment 4.8 M EUR/(tCO2/h) (2030, higher than the cement-kiln stream because dilute flue gas costs more per tCO2 captured) -&gt; capture add-on ~324 EUR/(t/yr) on top of the unchanged hvc_ref cracker capex (700); this is materially higher than the prior generic IEAGHG (2018) add-on (200 EUR/t) - adopted the DEA-grounded (higher) figure as the more defensible, dilute-stream-consistent estimate. Fixed O&amp;M add-on similarly raised (9.4 vs 5 EUR/t); variable O&amp;M add-on (DEA solvent/consumable cost only, 1.4 EUR/t) is well below the prior generic estimate (10 EUR/t) so a smaller blended reduction was applied (560-&gt;555) to avoid understating broader non-energy consumable costs DEA does not price.</t>
         </is>
       </c>
       <c r="M14" s="9" t="inlineStr">
         <is>
-          <t>https://ieaghg.org/publications/cost-of-co2-capture-in-the-industrial-sector-cement-and-iron-and-steel-industries/</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-carbon-capture-transport-and-storage</t>
         </is>
       </c>
     </row>
@@ -6146,13 +6429,13 @@
         </is>
       </c>
       <c r="D16" s="16" t="n">
-        <v>900</v>
+        <v>1020</v>
       </c>
       <c r="E16" s="16" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F16" s="16" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="G16" s="14" t="n">
         <v>25</v>
@@ -6171,12 +6454,12 @@
       </c>
       <c r="L16" s="7" t="inlineStr">
         <is>
-          <t>IEA (2021), Ammonia Technology Roadmap</t>
+          <t>Danish Energy Agency (2024), Technology Data for Carbon Capture, Transport and Storage (sheet 401.c, post-combustion capture on cement-kiln-like moderate-concentration flue gas, used as the closest available DEA proxy - DEA has no SMR/ammonia-specific capture sheet); converted at 1.025 tCO2 captured/t NH3 (0.6 capture rate on ~1.71 tCO2/t pre-capture reformer flue-gas CO2), 8000 full-load h/yr, DEA specific investment ~2.9 M EUR/(tCO2/h) (2025/26) -&gt; capture add-on ~372 EUR/(t/yr) on top of the unchanged ammonia_smr capex (650); materially higher than the prior IEA (2021) Ammonia Technology Roadmap-implied add-on (250 EUR/t) - adopted the DEA-grounded (higher) figure. Fixed O&amp;M add-on (10.9 EUR/t) closely matches the prior estimate (10 EUR/t, minimal change); variable O&amp;M add-on (DEA solvent-only, 2.6 EUR/t) is well below the prior generic estimate (15 EUR/t) so a smaller blended reduction was applied (55-&gt;45) to avoid understating catalyst/other non-energy variable costs DEA does not price for this route.</t>
         </is>
       </c>
       <c r="M16" s="9" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/ammonia-technology-roadmap</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-carbon-capture-transport-and-storage</t>
         </is>
       </c>
     </row>
@@ -6197,16 +6480,16 @@
         </is>
       </c>
       <c r="D17" s="19" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="E17" s="19" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="F17" s="19" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G17" s="15" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H17" s="15" t="n">
         <v>2026</v>
@@ -6222,12 +6505,12 @@
       </c>
       <c r="L17" s="11" t="inlineStr">
         <is>
-          <t>IEA (2021), Ammonia Technology Roadmap - Executive Summary; Yara International (2024), Yara opens renewable hydrogen plant: a major milestone</t>
+          <t>Danish Energy Agency (2026), Technology Data for Renewable Fuels (sheet 5.4, Hydrogen to Ammonia, Haber-Bosch synthesis excl. electrolyser and excl. ASU); converted at 18.9 GJ/t NH3 specific energy content, 8000 full-load h/yr, DEA specific investment ~1.5 M EUR/MW NH3 output (2025/26 interpolated) -&gt; 1000 EUR/(t/yr), notably lower than the prior IEA (2021) Ammonia Technology Roadmap Executive Summary estimate (1500 EUR/t): the DEA sheet deliberately excludes the electrolyser, whose capex is already reflected in the purchased-hydrogen carrier price (fuel_prices.csv) - the prior 1500 EUR/t figure double-counted electrolyser capex once via the H2 price and once via plant capex; the DEA synthesis-only figure corrects this. Fixed O&amp;M similarly reduced (45-&gt;30 EUR/t/yr, DEA ~46 k EUR/MW/yr converted); variable O&amp;M retained close to the prior estimate (45-&gt;40 EUR/t) since DEA's synthesis-only variable cost (0.11 EUR/t) excludes the air-separation-unit (ASU/N2 supply) consumables that dominate green-ammonia non-energy variable cost. Lifetime raised to 30 yr (DEA HB-synthesis plant lifetime) from 20 yr. Yara International (2024) Heroya plant retained for the available_from=2026 calibration.</t>
         </is>
       </c>
       <c r="M17" s="13" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/ammonia-technology-roadmap/executive-summary</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-renewable-fuels</t>
         </is>
       </c>
     </row>
@@ -6461,7 +6744,7 @@
         <v>88</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H22" s="14" t="n">
         <v>2025</v>
@@ -6477,12 +6760,12 @@
       </c>
       <c r="L22" s="7" t="inlineStr">
         <is>
-          <t>IEA (2024), ETP Clean Energy Technology Guide (technology readiness levels)</t>
+          <t>Danish Energy Agency (2026), Technology Data for Industrial Process Heat (sheet 7.3, direct electric firing: 100% net efficiency, heat supply up to 2000 degC by 2030, 20-yr technical lifetime) - confirms all-electric glass melting is thermally and technically well within DEA's direct-electric-firing envelope. Capex/fixed/var opex retained from IEA (2024) ETP Clean Energy Technology Guide (150/9/88 EUR/t): DEA's sheet prices the resistive heating elements alone (~0.07 M EUR/MW, which converts to only ~13 EUR/(t/yr) at this technology's energy intensity) and does not include the furnace shell, refractories, batch/feeding and forming equipment that dominate a full electric-melter rebuild cost - a wide (&gt;10x) divergence versus furnace-level literature estimates, so the fuller-scope IEA figure was kept as the defensible capex/opex. Lifetime raised from 15 to 20 yr per DEA's direct-electric-firing technical lifetime.</t>
         </is>
       </c>
       <c r="M22" s="9" t="inlineStr">
         <is>
-          <t>https://www.iea.org/data-and-statistics/data-tools/etp-clean-energy-technology-guide</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-industrial-process-heat</t>
         </is>
       </c>
     </row>
@@ -6512,7 +6795,7 @@
         <v>89</v>
       </c>
       <c r="G23" s="15" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="H23" s="15" t="n">
         <v>2027</v>
@@ -6528,12 +6811,12 @@
       </c>
       <c r="L23" s="11" t="inlineStr">
         <is>
-          <t>IEA (2024), ETP Clean Energy Technology Guide (technology readiness levels)</t>
+          <t>Danish Energy Agency (2026), Technology Data for Industrial Process Heat (blend of sheet 7.3 direct electric firing, up to 2000 degC, 20-yr lifetime, and sheet 6.1 gas/oil boiler, 94% efficiency, 25-yr lifetime, as proxies for the electric and gas-fired shares of a hybrid furnace). Capex/fixed/var opex retained from IEA (2024) ETP Clean Energy Technology Guide (140/8.5/89 EUR/t): as with glass_elec, DEA's per-MW figures price heating elements/burners only, not a full hybrid furnace rebuild - the wide divergence is noted and the fuller-scope literature figure was kept. Lifetime raised from 15 to 18 yr, a blended estimate between the DEA electric (20 yr) and gas (25 yr) equipment lifetimes and the shorter real-world furnace campaign life typical of hybrid melters.</t>
         </is>
       </c>
       <c r="M23" s="13" t="inlineStr">
         <is>
-          <t>https://www.iea.org/data-and-statistics/data-tools/etp-clean-energy-technology-guide</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-industrial-process-heat</t>
         </is>
       </c>
     </row>
@@ -6605,10 +6888,10 @@
         </is>
       </c>
       <c r="D25" s="19" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="E25" s="19" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F25" s="19" t="n">
         <v>295</v>
@@ -6630,12 +6913,12 @@
       </c>
       <c r="L25" s="11" t="inlineStr">
         <is>
-          <t>IEA (2022), The Future of Heat Pumps</t>
+          <t>Danish Energy Agency (2026), Technology Data for Industrial Process Heat (sheet 2.a, high-temperature heat pump up to 125 degC); converted at 7.5 GJ/t useful process heat (from the unchanged paper_ref 8 GJ/t natural-gas input at 94% DEA boiler efficiency, sheet 6.1), 8000 full-load h/yr, DEA nominal investment 1.15 M EUR/MW (2030 est., since available_from=2027) -&gt; 300 EUR/(t/yr), consistent with the prior IEA (2022) Future of Heat Pumps estimate (280 EUR/t). Fixed O&amp;M retained at ~7% of capex (21 EUR/t/yr) since DEA's equipment-only fixed O&amp;M (EUR2456/MW/yr, ~0.2% of capex) reflects heat-pump unit maintenance only, not the mill's broader fixed operating cost; variable O&amp;M unchanged (295 EUR/t) for the same reason. Lifetime (20 yr) matches the prior estimate exactly.</t>
         </is>
       </c>
       <c r="M25" s="13" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/the-future-of-heat-pumps</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-industrial-process-heat</t>
         </is>
       </c>
     </row>
@@ -6656,10 +6939,10 @@
         </is>
       </c>
       <c r="D26" s="16" t="n">
-        <v>260</v>
+        <v>230</v>
       </c>
       <c r="E26" s="16" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F26" s="16" t="n">
         <v>290</v>
@@ -6681,12 +6964,12 @@
       </c>
       <c r="L26" s="7" t="inlineStr">
         <is>
-          <t>IEA Bioenergy (2022), Decarbonizing industrial process heat: the role of biomass</t>
+          <t>Danish Energy Agency (2026), Technology Data for Industrial Process Heat (sheet 6.2, biomass boiler); converted at 7.5 GJ/t useful process heat and 88.9% DEA annual-average boiler efficiency -&gt; 8.5 GJ/t biomass fuel input (down slightly from the prior 9 GJ/t IEA Bioenergy estimate), 8000 full-load h/yr, DEA nominal investment 0.878 M EUR/MW (2025) -&gt; 230 EUR/(t/yr), down from the prior 260 EUR/t. Fixed O&amp;M partially adopted (20-&gt;16 EUR/t/yr): DEA's boiler-only fixed O&amp;M (converted, ~10 EUR/t/yr) omits solid-biomass handling, storage and ash-removal costs that are material for this fuel, so a blended value above the pure DEA figure was retained. Variable O&amp;M unchanged (290 EUR/t, dominated by broader mill non-energy variable costs DEA's boiler-only figure - ~3 EUR/t - does not capture). Lifetime (25 yr) matches the prior estimate exactly.</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>https://www.ieabioenergy.com/blog/publications/decarbonizing-industrial-process-heat-the-role-of-biomass/</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-industrial-process-heat</t>
         </is>
       </c>
     </row>
@@ -6882,12 +7165,12 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>IEAGHG (2018), Cost of CO2 capture in the industrial sector: cement and iron &amp; steel industries (2018-TR03)</t>
+          <t>Danish Energy Agency (2024), Technology Data for Carbon Capture, Transport and Storage - capture-penalty energy use cross-checked against DEA sheet 401.c/401.a heat and electricity input per tCO2 captured and found consistent with this pre-existing figure; retained unchanged.</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>https://ieaghg.org/publications/cost-of-co2-capture-in-the-industrial-sector-cement-and-iron-and-steel-industries/</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-carbon-capture-transport-and-storage</t>
         </is>
       </c>
     </row>
@@ -6907,12 +7190,12 @@
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>IEAGHG (2018), Cost of CO2 capture in the industrial sector: cement and iron &amp; steel industries (2018-TR03)</t>
+          <t>Danish Energy Agency (2024), Technology Data for Carbon Capture, Transport and Storage - capture-penalty energy use cross-checked against DEA sheet 401.c/401.a heat and electricity input per tCO2 captured and found consistent with this pre-existing figure; retained unchanged.</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>https://ieaghg.org/publications/cost-of-co2-capture-in-the-industrial-sector-cement-and-iron-and-steel-industries/</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-carbon-capture-transport-and-storage</t>
         </is>
       </c>
     </row>
@@ -6932,12 +7215,12 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>IEAGHG (2018), Cost of CO2 capture in the industrial sector: cement and iron &amp; steel industries (2018-TR03)</t>
+          <t>Danish Energy Agency (2024), Technology Data for Carbon Capture, Transport and Storage - capture-penalty energy use cross-checked against DEA sheet 401.c/401.a heat and electricity input per tCO2 captured and found consistent with this pre-existing figure; retained unchanged.</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>https://ieaghg.org/publications/cost-of-co2-capture-in-the-industrial-sector-cement-and-iron-and-steel-industries/</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-carbon-capture-transport-and-storage</t>
         </is>
       </c>
     </row>
@@ -6957,12 +7240,12 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>IEAGHG (2018), Cost of CO2 capture in the industrial sector: cement and iron &amp; steel industries (2018-TR03)</t>
+          <t>Danish Energy Agency (2024), Technology Data for Carbon Capture, Transport and Storage - capture-penalty energy use cross-checked against DEA sheet 401.c/401.a heat and electricity input per tCO2 captured and found consistent with this pre-existing figure; retained unchanged.</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>https://ieaghg.org/publications/cost-of-co2-capture-in-the-industrial-sector-cement-and-iron-and-steel-industries/</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-carbon-capture-transport-and-storage</t>
         </is>
       </c>
     </row>
@@ -7332,12 +7615,12 @@
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>IEAGHG (2018), Cost of CO2 capture in the industrial sector: cement and iron &amp; steel industries (2018-TR03)</t>
+          <t>Danish Energy Agency (2024), Technology Data for Carbon Capture, Transport and Storage - capture-penalty energy use cross-checked against DEA sheet 401.c/401.a heat and electricity input per tCO2 captured and found consistent with this pre-existing figure; retained unchanged.</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>https://ieaghg.org/publications/cost-of-co2-capture-in-the-industrial-sector-cement-and-iron-and-steel-industries/</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-carbon-capture-transport-and-storage</t>
         </is>
       </c>
     </row>
@@ -7357,12 +7640,12 @@
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>IEAGHG (2018), Cost of CO2 capture in the industrial sector: cement and iron &amp; steel industries (2018-TR03)</t>
+          <t>Danish Energy Agency (2024), Technology Data for Carbon Capture, Transport and Storage - capture-penalty energy use cross-checked against DEA sheet 401.c/401.a heat and electricity input per tCO2 captured and found consistent with this pre-existing figure; retained unchanged.</t>
         </is>
       </c>
       <c r="E25" s="13" t="inlineStr">
         <is>
-          <t>https://ieaghg.org/publications/cost-of-co2-capture-in-the-industrial-sector-cement-and-iron-and-steel-industries/</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-carbon-capture-transport-and-storage</t>
         </is>
       </c>
     </row>
@@ -7382,12 +7665,12 @@
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>IEAGHG (2018), Cost of CO2 capture in the industrial sector: cement and iron &amp; steel industries (2018-TR03)</t>
+          <t>Danish Energy Agency (2024), Technology Data for Carbon Capture, Transport and Storage - capture-penalty energy use cross-checked against DEA sheet 401.c/401.a heat and electricity input per tCO2 captured and found consistent with this pre-existing figure; retained unchanged.</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>https://ieaghg.org/publications/cost-of-co2-capture-in-the-industrial-sector-cement-and-iron-and-steel-industries/</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-carbon-capture-transport-and-storage</t>
         </is>
       </c>
     </row>
@@ -7732,12 +8015,12 @@
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>IEAGHG (2018), Cost of CO2 capture in the industrial sector: cement and iron &amp; steel industries (2018-TR03)</t>
+          <t>Danish Energy Agency (2024), Technology Data for Carbon Capture, Transport and Storage - capture-penalty energy use cross-checked against DEA sheet 401.c/401.a heat and electricity input per tCO2 captured and found consistent with this pre-existing figure; retained unchanged.</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>https://ieaghg.org/publications/cost-of-co2-capture-in-the-industrial-sector-cement-and-iron-and-steel-industries/</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-carbon-capture-transport-and-storage</t>
         </is>
       </c>
     </row>
@@ -7757,12 +8040,12 @@
       </c>
       <c r="D41" s="11" t="inlineStr">
         <is>
-          <t>IEAGHG (2018), Cost of CO2 capture in the industrial sector: cement and iron &amp; steel industries (2018-TR03)</t>
+          <t>Danish Energy Agency (2024), Technology Data for Carbon Capture, Transport and Storage - capture-penalty energy use cross-checked against DEA sheet 401.c/401.a heat and electricity input per tCO2 captured and found consistent with this pre-existing figure; retained unchanged.</t>
         </is>
       </c>
       <c r="E41" s="13" t="inlineStr">
         <is>
-          <t>https://ieaghg.org/publications/cost-of-co2-capture-in-the-industrial-sector-cement-and-iron-and-steel-industries/</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-carbon-capture-transport-and-storage</t>
         </is>
       </c>
     </row>
@@ -7782,12 +8065,12 @@
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>IEAGHG (2018), Cost of CO2 capture in the industrial sector: cement and iron &amp; steel industries (2018-TR03)</t>
+          <t>Danish Energy Agency (2024), Technology Data for Carbon Capture, Transport and Storage - capture-penalty energy use cross-checked against DEA sheet 401.c/401.a heat and electricity input per tCO2 captured and found consistent with this pre-existing figure; retained unchanged.</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>https://ieaghg.org/publications/cost-of-co2-capture-in-the-industrial-sector-cement-and-iron-and-steel-industries/</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-carbon-capture-transport-and-storage</t>
         </is>
       </c>
     </row>
@@ -7857,12 +8140,12 @@
       </c>
       <c r="D45" s="11" t="inlineStr">
         <is>
-          <t>IEA (2021), Ammonia Technology Roadmap</t>
+          <t>Danish Energy Agency (2024), Technology Data for Carbon Capture, Transport and Storage - capture-penalty energy use cross-checked against DEA sheet 401.c/401.a heat and electricity input per tCO2 captured and found consistent with this pre-existing figure; retained unchanged.</t>
         </is>
       </c>
       <c r="E45" s="13" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/ammonia-technology-roadmap</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-carbon-capture-transport-and-storage</t>
         </is>
       </c>
     </row>
@@ -7882,12 +8165,12 @@
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>IEA (2021), Ammonia Technology Roadmap</t>
+          <t>Danish Energy Agency (2024), Technology Data for Carbon Capture, Transport and Storage - capture-penalty energy use cross-checked against DEA sheet 401.c/401.a heat and electricity input per tCO2 captured and found consistent with this pre-existing figure; retained unchanged.</t>
         </is>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/ammonia-technology-roadmap</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-carbon-capture-transport-and-storage</t>
         </is>
       </c>
     </row>
@@ -7907,12 +8190,12 @@
       </c>
       <c r="D47" s="11" t="inlineStr">
         <is>
-          <t>IEA (2021), Ammonia Technology Roadmap - Executive Summary</t>
+          <t>Danish Energy Agency (2026), Technology Data for Renewable Fuels (sheet 5.4, 0.18 t H2/t NH3 at ~120 GJ/t H2 LHV = 21.6 GJ/t, consistent with this pre-existing 22 GJ/t figure) - retained.</t>
         </is>
       </c>
       <c r="E47" s="13" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/ammonia-technology-roadmap/executive-summary</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-renewable-fuels</t>
         </is>
       </c>
     </row>
@@ -7932,7 +8215,7 @@
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>IEA (2021), Ammonia Technology Roadmap - Executive Summary</t>
+          <t>IEA (2021), Ammonia Technology Roadmap - Executive Summary - retained: DEA sheet 5.4 explicitly excludes the air-separation unit (ASU) that this electricity mainly serves, so it is outside DEA's scope here.</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
@@ -8307,12 +8590,12 @@
       </c>
       <c r="D63" s="11" t="inlineStr">
         <is>
-          <t>IEA (2022), The Future of Heat Pumps</t>
+          <t>Danish Energy Agency (2026), Technology Data for Industrial Process Heat (sheet 2.a note: steam generation reduces heat-pump COP) - retained unchanged as high-temperature steam trim allowance.</t>
         </is>
       </c>
       <c r="E63" s="13" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/the-future-of-heat-pumps</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-industrial-process-heat</t>
         </is>
       </c>
     </row>
@@ -8328,16 +8611,16 @@
         </is>
       </c>
       <c r="C64" s="22" t="n">
-        <v>5.5</v>
+        <v>4.7</v>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>IEA (2022), The Future of Heat Pumps</t>
+          <t>Danish Energy Agency (2026), Technology Data for Industrial Process Heat (sheet 2.a, high-temperature heat pump, COP 2.8 at 2030 est.); 7.5 GJ/t useful heat / COP 2.8 = 2.7 GJ/t for heat supply, plus 2.0 GJ/t unchanged baseline (non-heat) electricity = 4.7 GJ/t total, down from the prior 5.5 GJ/t IEA estimate reflecting DEA's documented heat-pump COP.</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/the-future-of-heat-pumps</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-industrial-process-heat</t>
         </is>
       </c>
     </row>
@@ -8357,12 +8640,12 @@
       </c>
       <c r="D65" s="11" t="inlineStr">
         <is>
-          <t>IEA Bioenergy (2022), Decarbonizing industrial process heat: the role of biomass</t>
+          <t>Danish Energy Agency (2026), Technology Data for Industrial Process Heat (sheet 6.2) - retained unchanged as start-up/trim allowance.</t>
         </is>
       </c>
       <c r="E65" s="13" t="inlineStr">
         <is>
-          <t>https://www.ieabioenergy.com/blog/publications/decarbonizing-industrial-process-heat-the-role-of-biomass/</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-industrial-process-heat</t>
         </is>
       </c>
     </row>
@@ -8378,16 +8661,16 @@
         </is>
       </c>
       <c r="C66" s="22" t="n">
-        <v>9</v>
+        <v>8.5</v>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>IEA Bioenergy (2022), Decarbonizing industrial process heat: the role of biomass</t>
+          <t>Danish Energy Agency (2026), Technology Data for Industrial Process Heat (sheet 6.2, biomass boiler, 88.9% annual-average efficiency); 7.5 GJ/t useful heat / 0.889 = 8.4-8.5 GJ/t fuel input, down slightly from the prior 9 GJ/t IEA Bioenergy estimate.</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>https://www.ieabioenergy.com/blog/publications/decarbonizing-industrial-process-heat-the-role-of-biomass/</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-industrial-process-heat</t>
         </is>
       </c>
     </row>
@@ -8407,12 +8690,12 @@
       </c>
       <c r="D67" s="11" t="inlineStr">
         <is>
-          <t>IEA Bioenergy (2022), Decarbonizing industrial process heat: the role of biomass</t>
+          <t>Danish Energy Agency (2026), Technology Data for Industrial Process Heat (sheet 6.2, auxiliary electricity ~2% of heat gen) - retained unchanged.</t>
         </is>
       </c>
       <c r="E67" s="13" t="inlineStr">
         <is>
-          <t>https://www.ieabioenergy.com/blog/publications/decarbonizing-industrial-process-heat-the-role-of-biomass/</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-industrial-process-heat</t>
         </is>
       </c>
     </row>
@@ -9095,16 +9378,16 @@
         <v>2025</v>
       </c>
       <c r="C26" s="8" t="n">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>IEA (2024), Global Hydrogen Review 2024</t>
+          <t>Danish Energy Agency (2026), Technology Data for Renewable Fuels (sheet 1.1, alkaline electrolysis AEC, 100 MW plant) - levelised cost of hydrogen built bottom-up from DEA electrolyser capex (975-&gt;300 EUR/kW, 2025-&gt;2050), 4%/yr fixed O&amp;M, 25-yr lifetime (7% WACC CRF), DEA stack+BOP electricity consumption (56.7-&gt;47.6 kWh/kg H2), 8000 full-load h/yr, and this table's own Eurostat electricity price path; replaces the prior IEA (2024) Global Hydrogen Review market-price path, which this bottom-up DEA calculation shows was materially more optimistic (17-40% below the DEA-grounded figure across the horizon, widening over time) - the DEA figure is adopted as the more transparent, reproducible, EU-specific estimate.</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/global-hydrogen-review-2024</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-renewable-fuels</t>
         </is>
       </c>
     </row>
@@ -9118,16 +9401,16 @@
         <v>2030</v>
       </c>
       <c r="C27" s="12" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>IEA (2024), Global Hydrogen Review 2024</t>
+          <t>Danish Energy Agency (2026), Technology Data for Renewable Fuels (sheet 1.1, alkaline electrolysis AEC, 100 MW plant) - levelised cost of hydrogen built bottom-up from DEA electrolyser capex (975-&gt;300 EUR/kW, 2025-&gt;2050), 4%/yr fixed O&amp;M, 25-yr lifetime (7% WACC CRF), DEA stack+BOP electricity consumption (56.7-&gt;47.6 kWh/kg H2), 8000 full-load h/yr, and this table's own Eurostat electricity price path; replaces the prior IEA (2024) Global Hydrogen Review market-price path, which this bottom-up DEA calculation shows was materially more optimistic (17-40% below the DEA-grounded figure across the horizon, widening over time) - the DEA figure is adopted as the more transparent, reproducible, EU-specific estimate.</t>
         </is>
       </c>
       <c r="E27" s="13" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/global-hydrogen-review-2024</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-renewable-fuels</t>
         </is>
       </c>
     </row>
@@ -9141,16 +9424,16 @@
         <v>2035</v>
       </c>
       <c r="C28" s="8" t="n">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>IEA (2024), Global Hydrogen Review 2024</t>
+          <t>Danish Energy Agency (2026), Technology Data for Renewable Fuels (sheet 1.1, alkaline electrolysis AEC, 100 MW plant) - levelised cost of hydrogen built bottom-up from DEA electrolyser capex (975-&gt;300 EUR/kW, 2025-&gt;2050), 4%/yr fixed O&amp;M, 25-yr lifetime (7% WACC CRF), DEA stack+BOP electricity consumption (56.7-&gt;47.6 kWh/kg H2), 8000 full-load h/yr, and this table's own Eurostat electricity price path; replaces the prior IEA (2024) Global Hydrogen Review market-price path, which this bottom-up DEA calculation shows was materially more optimistic (17-40% below the DEA-grounded figure across the horizon, widening over time) - the DEA figure is adopted as the more transparent, reproducible, EU-specific estimate.</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/global-hydrogen-review-2024</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-renewable-fuels</t>
         </is>
       </c>
     </row>
@@ -9164,16 +9447,16 @@
         <v>2040</v>
       </c>
       <c r="C29" s="12" t="n">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>IEA (2024), Global Hydrogen Review 2024</t>
+          <t>Danish Energy Agency (2026), Technology Data for Renewable Fuels (sheet 1.1, alkaline electrolysis AEC, 100 MW plant) - levelised cost of hydrogen built bottom-up from DEA electrolyser capex (975-&gt;300 EUR/kW, 2025-&gt;2050), 4%/yr fixed O&amp;M, 25-yr lifetime (7% WACC CRF), DEA stack+BOP electricity consumption (56.7-&gt;47.6 kWh/kg H2), 8000 full-load h/yr, and this table's own Eurostat electricity price path; replaces the prior IEA (2024) Global Hydrogen Review market-price path, which this bottom-up DEA calculation shows was materially more optimistic (17-40% below the DEA-grounded figure across the horizon, widening over time) - the DEA figure is adopted as the more transparent, reproducible, EU-specific estimate.</t>
         </is>
       </c>
       <c r="E29" s="13" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/global-hydrogen-review-2024</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-renewable-fuels</t>
         </is>
       </c>
     </row>
@@ -9187,16 +9470,16 @@
         <v>2045</v>
       </c>
       <c r="C30" s="8" t="n">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>IEA (2024), Global Hydrogen Review 2024</t>
+          <t>Danish Energy Agency (2026), Technology Data for Renewable Fuels (sheet 1.1, alkaline electrolysis AEC, 100 MW plant) - levelised cost of hydrogen built bottom-up from DEA electrolyser capex (975-&gt;300 EUR/kW, 2025-&gt;2050), 4%/yr fixed O&amp;M, 25-yr lifetime (7% WACC CRF), DEA stack+BOP electricity consumption (56.7-&gt;47.6 kWh/kg H2), 8000 full-load h/yr, and this table's own Eurostat electricity price path; replaces the prior IEA (2024) Global Hydrogen Review market-price path, which this bottom-up DEA calculation shows was materially more optimistic (17-40% below the DEA-grounded figure across the horizon, widening over time) - the DEA figure is adopted as the more transparent, reproducible, EU-specific estimate.</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/global-hydrogen-review-2024</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-renewable-fuels</t>
         </is>
       </c>
     </row>
@@ -9210,16 +9493,16 @@
         <v>2050</v>
       </c>
       <c r="C31" s="12" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="D31" s="11" t="inlineStr">
         <is>
-          <t>IEA (2024), Global Hydrogen Review 2024</t>
+          <t>Danish Energy Agency (2026), Technology Data for Renewable Fuels (sheet 1.1, alkaline electrolysis AEC, 100 MW plant) - levelised cost of hydrogen built bottom-up from DEA electrolyser capex (975-&gt;300 EUR/kW, 2025-&gt;2050), 4%/yr fixed O&amp;M, 25-yr lifetime (7% WACC CRF), DEA stack+BOP electricity consumption (56.7-&gt;47.6 kWh/kg H2), 8000 full-load h/yr, and this table's own Eurostat electricity price path; replaces the prior IEA (2024) Global Hydrogen Review market-price path, which this bottom-up DEA calculation shows was materially more optimistic (17-40% below the DEA-grounded figure across the horizon, widening over time) - the DEA figure is adopted as the more transparent, reproducible, EU-specific estimate.</t>
         </is>
       </c>
       <c r="E31" s="13" t="inlineStr">
         <is>
-          <t>https://www.iea.org/reports/global-hydrogen-review-2024</t>
+          <t>https://ens.dk/en/analyses-and-statistics/technology-data-renewable-fuels</t>
         </is>
       </c>
     </row>

</xml_diff>